<commit_message>
sensitivity analysis - not good
</commit_message>
<xml_diff>
--- a/simulatedData/dataset_hypothetical.xlsx
+++ b/simulatedData/dataset_hypothetical.xlsx
@@ -492,7 +492,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>5.512980572083857e-12</v>
+        <v>5.443484845281919e-12</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
@@ -504,28 +504,28 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9.699347069291397</v>
+        <v>9.699347069291393</v>
       </c>
       <c r="F2" t="n">
-        <v>4.985069224042763</v>
+        <v>4.985069224042767</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>2.69743038542935</v>
+        <v>2.697430405916348</v>
       </c>
       <c r="I2" t="n">
-        <v>50.0993034714063</v>
+        <v>50.0993040483645</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>3.092067173384319</v>
+        <v>3.092067302409011</v>
       </c>
       <c r="L2" t="n">
-        <v>25.25641044512075</v>
+        <v>25.25640953197178</v>
       </c>
     </row>
     <row r="3">
@@ -542,28 +542,28 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>9.63035488551003</v>
+        <v>9.630354885510028</v>
       </c>
       <c r="F3" t="n">
-        <v>5.020873794760699</v>
+        <v>5.020873794760672</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>2.758249423216762</v>
+        <v>2.758249353703567</v>
       </c>
       <c r="I3" t="n">
-        <v>48.61131297180568</v>
+        <v>48.61131064316509</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>3.176064831617197</v>
+        <v>3.176064903438797</v>
       </c>
       <c r="L3" t="n">
-        <v>24.5436117665439</v>
+        <v>24.54361124311865</v>
       </c>
     </row>
     <row r="4">
@@ -583,25 +583,25 @@
         <v>9.560827209729428</v>
       </c>
       <c r="F4" t="n">
-        <v>5.057481072452409</v>
+        <v>5.057481072452389</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>2.82085533822959</v>
+        <v>2.820855337202761</v>
       </c>
       <c r="I4" t="n">
-        <v>47.18827644611995</v>
+        <v>47.18827641641769</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>3.260709249356306</v>
+        <v>3.260709315896745</v>
       </c>
       <c r="L4" t="n">
-        <v>23.86623886383631</v>
+        <v>23.86623840568347</v>
       </c>
     </row>
     <row r="5">
@@ -621,25 +621,25 @@
         <v>9.490772943835177</v>
       </c>
       <c r="F5" t="n">
-        <v>5.094910212584622</v>
+        <v>5.094910212584586</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>2.885113010565214</v>
+        <v>2.88511300332616</v>
       </c>
       <c r="I5" t="n">
-        <v>45.82807871494958</v>
+        <v>45.82807847675473</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>3.345941090590222</v>
+        <v>3.345941141093194</v>
       </c>
       <c r="L5" t="n">
-        <v>23.22209150109784</v>
+        <v>23.22209118380449</v>
       </c>
     </row>
     <row r="6">
@@ -656,28 +656,28 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>9.420201171386378</v>
+        <v>9.420201171386379</v>
       </c>
       <c r="F6" t="n">
-        <v>5.133180979166142</v>
+        <v>5.133180979166139</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>2.950892882690657</v>
+        <v>2.950892880225108</v>
       </c>
       <c r="I6" t="n">
-        <v>44.5284663082974</v>
+        <v>44.52846622806055</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3.431702821871986</v>
+        <v>3.431702862494683</v>
       </c>
       <c r="L6" t="n">
-        <v>22.60912863329828</v>
+        <v>22.60912837113162</v>
       </c>
     </row>
     <row r="7">
@@ -694,28 +694,28 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>9.349121163616877</v>
+        <v>9.349121163616873</v>
       </c>
       <c r="F7" t="n">
-        <v>5.172313763739869</v>
+        <v>5.172313763739848</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>3.018070959187208</v>
+        <v>3.01807095925132</v>
       </c>
       <c r="I7" t="n">
-        <v>43.2870928103194</v>
+        <v>43.28709281230567</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>3.517939749213151</v>
+        <v>3.517939746769324</v>
       </c>
       <c r="L7" t="n">
-        <v>22.02544939518506</v>
+        <v>22.02544941102833</v>
       </c>
     </row>
     <row r="8">
@@ -732,33 +732,33 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>9.277542385800684</v>
+        <v>9.277542385800682</v>
       </c>
       <c r="F8" t="n">
-        <v>5.21232960476861</v>
+        <v>5.212329604768589</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>3.086528906612338</v>
+        <v>3.086528906879938</v>
       </c>
       <c r="I8" t="n">
-        <v>42.10156260324491</v>
+        <v>42.10156261211326</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>3.604599176807855</v>
+        <v>3.604599169038484</v>
       </c>
       <c r="L8" t="n">
-        <v>21.46928765764942</v>
+        <v>21.46928770458955</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1.615375460547206e-11</v>
+        <v>4.771601926726869e-12</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -770,33 +770,33 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>9.205474504005355</v>
+        <v>9.205474504005354</v>
       </c>
       <c r="F9" t="n">
-        <v>5.253250207385433</v>
+        <v>5.253250207385437</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>3.156153512598828</v>
+        <v>3.156153997553547</v>
       </c>
       <c r="I9" t="n">
-        <v>40.9694764901717</v>
+        <v>40.96946516035371</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>3.691630534726485</v>
+        <v>3.691630532625133</v>
       </c>
       <c r="L9" t="n">
-        <v>20.93900050172503</v>
+        <v>20.93900051358815</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.611868224115192e-11</v>
+        <v>4.757130086568783e-12</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -811,30 +811,30 @@
         <v>9.132927392258562</v>
       </c>
       <c r="F10" t="n">
-        <v>5.295097963471854</v>
+        <v>5.295097963471852</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>3.226838708796441</v>
+        <v>3.226839002257657</v>
       </c>
       <c r="I10" t="n">
-        <v>39.88840949574709</v>
+        <v>39.88840321610132</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>3.778985064195272</v>
+        <v>3.778985068429549</v>
       </c>
       <c r="L10" t="n">
-        <v>20.43306025874206</v>
+        <v>20.43306023696256</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4.740829331029515e-12</v>
+        <v>1.607854903206587e-11</v>
       </c>
       <c r="B11" t="n">
         <v>0</v>
@@ -849,25 +849,25 @@
         <v>9.059911140154993</v>
       </c>
       <c r="F11" t="n">
-        <v>5.337895972019203</v>
+        <v>5.337895972019213</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>3.298482028508494</v>
+        <v>3.298481770332996</v>
       </c>
       <c r="I11" t="n">
-        <v>38.85601511690004</v>
+        <v>38.85602027941138</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>3.866615747698372</v>
+        <v>3.866615740128793</v>
       </c>
       <c r="L11" t="n">
-        <v>19.95004562846234</v>
+        <v>19.9500456629309</v>
       </c>
     </row>
     <row r="12">
@@ -884,28 +884,28 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>8.986436060932464</v>
+        <v>8.986436060932469</v>
       </c>
       <c r="F12" t="n">
-        <v>5.381668059720168</v>
+        <v>5.38166805972018</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>3.370986326462548</v>
+        <v>3.370986326460237</v>
       </c>
       <c r="I12" t="n">
-        <v>37.8699922225055</v>
+        <v>37.86999222242693</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>3.954477138722531</v>
+        <v>3.954477139618122</v>
       </c>
       <c r="L12" t="n">
-        <v>19.48863399885695</v>
+        <v>19.48863399476637</v>
       </c>
     </row>
     <row r="13">
@@ -925,25 +925,25 @@
         <v>8.912512700048374</v>
       </c>
       <c r="F13" t="n">
-        <v>5.426438801725505</v>
+        <v>5.426438801725501</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>3.444260067875105</v>
+        <v>3.444260067874878</v>
       </c>
       <c r="I13" t="n">
-        <v>36.92809202184588</v>
+        <v>36.92809202183857</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>4.042525290505201</v>
+        <v>4.042525290504308</v>
       </c>
       <c r="L13" t="n">
-        <v>19.04759385653467</v>
+        <v>19.0475938565376</v>
       </c>
     </row>
     <row r="14">
@@ -960,33 +960,33 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>8.838151844289545</v>
+        <v>8.838151844289541</v>
       </c>
       <c r="F14" t="n">
-        <v>5.47223354249082</v>
+        <v>5.472233542490808</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3.51821573641599</v>
+        <v>3.518216099303301</v>
       </c>
       <c r="I14" t="n">
-        <v>36.02815393731253</v>
+        <v>36.02814793334121</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>4.130717623279303</v>
+        <v>4.130717622989087</v>
       </c>
       <c r="L14" t="n">
-        <v>18.62577808350046</v>
+        <v>18.62577808474621</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1.586863780719597e-11</v>
+        <v>4.657786957480437e-12</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -998,33 +998,33 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>8.763364531451209</v>
+        <v>8.763364531451213</v>
       </c>
       <c r="F15" t="n">
-        <v>5.519078416623445</v>
+        <v>5.519078416623477</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>3.592771068345179</v>
+        <v>3.592771760862532</v>
       </c>
       <c r="I15" t="n">
-        <v>35.16808564140039</v>
+        <v>35.16807492260258</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>4.219012847189298</v>
+        <v>4.219012847104465</v>
       </c>
       <c r="L15" t="n">
-        <v>18.22211753388449</v>
+        <v>18.22211753419642</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>4.632685396169775e-12</v>
+        <v>1.580413030208249e-11</v>
       </c>
       <c r="B16" t="n">
         <v>0</v>
@@ -1036,28 +1036,28 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>8.688162060623027</v>
+        <v>8.688162060623023</v>
       </c>
       <c r="F16" t="n">
-        <v>5.567000369624424</v>
+        <v>5.567000369624425</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>3.667848520867208</v>
+        <v>3.667848486320693</v>
       </c>
       <c r="I16" t="n">
-        <v>34.34587579881062</v>
+        <v>34.34587631889599</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>4.307370868128792</v>
+        <v>4.307370868235205</v>
       </c>
       <c r="L16" t="n">
-        <v>17.83561520763794</v>
+        <v>17.83561520735162</v>
       </c>
     </row>
     <row r="17">
@@ -1074,28 +1074,28 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>8.612556003123021</v>
+        <v>8.61255600312302</v>
       </c>
       <c r="F17" t="n">
-        <v>5.616027178402847</v>
+        <v>5.616027178402867</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3.743371842357093</v>
+        <v>3.743371850910907</v>
       </c>
       <c r="I17" t="n">
-        <v>33.55964164941631</v>
+        <v>33.55964152193394</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>4.395752719513276</v>
+        <v>4.395752719586175</v>
       </c>
       <c r="L17" t="n">
-        <v>17.46534079616599</v>
+        <v>17.46534079596972</v>
       </c>
     </row>
     <row r="18">
@@ -1112,28 +1112,28 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>8.53655821412304</v>
+        <v>8.536558214123042</v>
       </c>
       <c r="F18" t="n">
-        <v>5.666187471420748</v>
+        <v>5.666187471420737</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>3.819270954890266</v>
+        <v>3.819270939230787</v>
       </c>
       <c r="I18" t="n">
-        <v>32.80755260969687</v>
+        <v>32.80755282507882</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>4.484120483205356</v>
+        <v>4.484120482968211</v>
       </c>
       <c r="L18" t="n">
-        <v>17.11042571753297</v>
+        <v>17.11042571830219</v>
       </c>
     </row>
     <row r="19">
@@ -1150,28 +1150,28 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>8.460180845012575</v>
+        <v>8.460180845012571</v>
       </c>
       <c r="F19" t="n">
-        <v>5.717510748302256</v>
+        <v>5.717510748302229</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>3.895478511670832</v>
+        <v>3.895478513272141</v>
       </c>
       <c r="I19" t="n">
-        <v>32.08787906372914</v>
+        <v>32.08787904216323</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>4.57243723482427</v>
+        <v>4.572437234826272</v>
       </c>
       <c r="L19" t="n">
-        <v>16.77005847775977</v>
+        <v>16.77005847775497</v>
       </c>
     </row>
     <row r="20">
@@ -1188,28 +1188,28 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>8.383436356550771</v>
+        <v>8.383436356550773</v>
       </c>
       <c r="F20" t="n">
-        <v>5.770027398716886</v>
+        <v>5.770027398716848</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>3.971930492949263</v>
+        <v>3.971930492951591</v>
       </c>
       <c r="I20" t="n">
-        <v>31.39897843768169</v>
+        <v>31.39897843765132</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>4.660666984006019</v>
+        <v>4.660666984094037</v>
       </c>
       <c r="L20" t="n">
-        <v>16.44348043496179</v>
+        <v>16.44348043465661</v>
       </c>
     </row>
     <row r="21">
@@ -1229,25 +1229,25 @@
         <v>8.30633753286056</v>
       </c>
       <c r="F21" t="n">
-        <v>5.823768720316768</v>
+        <v>5.823768720316807</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>4.048565931560494</v>
+        <v>4.048565932038013</v>
       </c>
       <c r="I21" t="n">
-        <v>30.73929403167219</v>
+        <v>30.73929402712836</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>4.748774623882341</v>
+        <v>4.74877462388235</v>
       </c>
       <c r="L21" t="n">
-        <v>16.12998188670693</v>
+        <v>16.12998188670748</v>
       </c>
     </row>
     <row r="22">
@@ -1264,28 +1264,28 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>8.228897496322057</v>
+        <v>8.228897496322054</v>
       </c>
       <c r="F22" t="n">
-        <v>5.878766935474659</v>
+        <v>5.8787669354746</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>4.125326703088624</v>
+        <v>4.125326786189955</v>
       </c>
       <c r="I22" t="n">
-        <v>30.10735244292725</v>
+        <v>30.10735151929713</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>4.836725883699709</v>
+        <v>4.836725883699718</v>
       </c>
       <c r="L22" t="n">
-        <v>15.82889847330952</v>
+        <v>15.82889847330988</v>
       </c>
     </row>
     <row r="23">
@@ -1305,25 +1305,25 @@
         <v>8.151129723426582</v>
       </c>
       <c r="F23" t="n">
-        <v>5.935055206531888</v>
+        <v>5.935055206531922</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>4.202157642877698</v>
+        <v>4.202157636599373</v>
       </c>
       <c r="I23" t="n">
-        <v>29.50175727088129</v>
+        <v>29.50175733780496</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>4.924487287408027</v>
+        <v>4.924487287391338</v>
       </c>
       <c r="L23" t="n">
-        <v>15.53960786203673</v>
+        <v>15.53960786209036</v>
       </c>
     </row>
     <row r="24">
@@ -1340,28 +1340,28 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>8.073048061657222</v>
+        <v>8.073048061657223</v>
       </c>
       <c r="F24" t="n">
-        <v>5.992667649224881</v>
+        <v>5.992667649224857</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>4.279005677896204</v>
+        <v>4.279005674422212</v>
       </c>
       <c r="I24" t="n">
-        <v>28.92119351470508</v>
+        <v>28.92119355072527</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>5.01202611496033</v>
+        <v>5.012026114971531</v>
       </c>
       <c r="L24" t="n">
-        <v>15.261526698943</v>
+        <v>15.26152669890068</v>
       </c>
     </row>
     <row r="25">
@@ -1378,28 +1378,28 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>7.994666747465937</v>
+        <v>7.994666747465935</v>
       </c>
       <c r="F25" t="n">
-        <v>6.051639343908534</v>
+        <v>6.051639343908493</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>4.355820388122174</v>
+        <v>4.355820387296889</v>
       </c>
       <c r="I25" t="n">
-        <v>28.36441613992006</v>
+        <v>28.3644161481989</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>5.099310367626974</v>
+        <v>5.099310367635607</v>
       </c>
       <c r="L25" t="n">
-        <v>14.99410780128293</v>
+        <v>14.99410780125049</v>
       </c>
     </row>
     <row r="26">
@@ -1416,28 +1416,28 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>7.916000425422451</v>
+        <v>7.916000425422448</v>
       </c>
       <c r="F26" t="n">
-        <v>6.112006344143049</v>
+        <v>6.112006344143065</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>4.432553509000461</v>
+        <v>4.432553505047626</v>
       </c>
       <c r="I26" t="n">
-        <v>27.83025045929205</v>
+        <v>27.83025049707959</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>5.186308736296866</v>
+        <v>5.186308736294465</v>
       </c>
       <c r="L26" t="n">
-        <v>14.73683757299216</v>
+        <v>14.73683757300254</v>
       </c>
     </row>
     <row r="27">
@@ -1454,28 +1454,28 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>7.837064168615009</v>
+        <v>7.837064168615004</v>
       </c>
       <c r="F27" t="n">
-        <v>6.173805682149561</v>
+        <v>6.173805682149499</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>4.509158846922761</v>
+        <v>4.509158846994181</v>
       </c>
       <c r="I27" t="n">
-        <v>27.31758801190363</v>
+        <v>27.31758801123689</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>5.272990572696988</v>
+        <v>5.27299057269192</v>
       </c>
       <c r="L27" t="n">
-        <v>14.48923362418039</v>
+        <v>14.48923362419971</v>
       </c>
     </row>
     <row r="28">
@@ -1492,28 +1492,28 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>7.757873500388881</v>
+        <v>7.757873500388883</v>
       </c>
       <c r="F28" t="n">
-        <v>6.23707537056989</v>
+        <v>6.237075370569893</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>4.585592154086891</v>
+        <v>4.585592156148826</v>
       </c>
       <c r="I28" t="n">
-        <v>26.82538304788634</v>
+        <v>26.82538302991853</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>5.359325863194083</v>
+        <v>5.359325863191454</v>
       </c>
       <c r="L28" t="n">
-        <v>14.25084257790937</v>
+        <v>14.25084257792133</v>
       </c>
     </row>
     <row r="29">
@@ -1530,28 +1530,28 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>7.678444417513585</v>
+        <v>7.678444417513592</v>
       </c>
       <c r="F29" t="n">
-        <v>6.301854399891663</v>
+        <v>6.301854399891735</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>4.661811018407692</v>
+        <v>4.661811017948281</v>
       </c>
       <c r="I29" t="n">
-        <v>26.35264904849958</v>
+        <v>26.35264905238753</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>5.445285204849962</v>
+        <v>5.445285204849969</v>
       </c>
       <c r="L29" t="n">
-        <v>14.02123804899962</v>
+        <v>14.02123804899875</v>
       </c>
     </row>
     <row r="30">
@@ -1571,25 +1571,25 @@
         <v>7.598793414876552</v>
       </c>
       <c r="F30" t="n">
-        <v>6.368182730810259</v>
+        <v>6.368182730810237</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4.737774732483755</v>
+        <v>4.737774732130628</v>
       </c>
       <c r="I30" t="n">
-        <v>25.89845560569227</v>
+        <v>25.8984556086091</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>5.530839783609424</v>
+        <v>5.530839783609429</v>
       </c>
       <c r="L30" t="n">
-        <v>13.80001878022639</v>
+        <v>13.8000187802265</v>
       </c>
     </row>
     <row r="31">
@@ -1609,30 +1609,30 @@
         <v>7.518937511806604</v>
       </c>
       <c r="F31" t="n">
-        <v>6.436101280702517</v>
+        <v>6.436101280702531</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>4.813444211282237</v>
+        <v>4.813444211286638</v>
       </c>
       <c r="I31" t="n">
-        <v>25.46192506409847</v>
+        <v>25.46192506406228</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>5.615961354369177</v>
+        <v>5.615961354369178</v>
       </c>
       <c r="L31" t="n">
-        <v>13.58680692298745</v>
+        <v>13.58680692298771</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1.418159695979697e-11</v>
+        <v>8.937688241234482e-12</v>
       </c>
       <c r="B32" t="n">
         <v>0</v>
@@ -1644,33 +1644,33 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>7.43889428013757</v>
+        <v>7.438894280137573</v>
       </c>
       <c r="F32" t="n">
-        <v>6.505651903280182</v>
+        <v>6.505651903280183</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>4.888781886760984</v>
+        <v>4.888781886761088</v>
       </c>
       <c r="I32" t="n">
-        <v>25.04222956274659</v>
+        <v>25.04222956274972</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>5.700622222755028</v>
+        <v>5.70062222275502</v>
       </c>
       <c r="L32" t="n">
-        <v>13.38124645038788</v>
+        <v>13.3812464503874</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.2416149156737015</v>
+        <v>0.241614915920489</v>
       </c>
       <c r="B33" t="n">
         <v>0</v>
@@ -1682,33 +1682,33 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>7.358681874128892</v>
+        <v>7.358681874128894</v>
       </c>
       <c r="F33" t="n">
-        <v>6.576877360362939</v>
+        <v>6.576877360362941</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>4.960086384449329</v>
+        <v>4.960086384437963</v>
       </c>
       <c r="I33" t="n">
-        <v>24.65800819910117</v>
+        <v>24.6580081992406</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>5.784795228444019</v>
+        <v>5.784795228443813</v>
       </c>
       <c r="L33" t="n">
-        <v>13.18300169178787</v>
+        <v>13.18300169179237</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.545486432314442</v>
+        <v>0.5454864322902875</v>
       </c>
       <c r="B34" t="n">
         <v>0</v>
@@ -1720,33 +1720,33 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>7.278319062367192</v>
+        <v>7.278319062367198</v>
       </c>
       <c r="F34" t="n">
-        <v>6.649821284579757</v>
+        <v>6.649821284579734</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>5.02997695411799</v>
+        <v>5.029976954118224</v>
       </c>
       <c r="I34" t="n">
-        <v>24.29307441699436</v>
+        <v>24.29307441699305</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>5.868453729884763</v>
+        <v>5.868453729884766</v>
       </c>
       <c r="L34" t="n">
-        <v>12.9917559787475</v>
+        <v>12.99175597874675</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.8714397698282672</v>
+        <v>0.8714397699293456</v>
       </c>
       <c r="B35" t="n">
         <v>0</v>
@@ -1761,30 +1761,30 @@
         <v>7.197825261779796</v>
       </c>
       <c r="F35" t="n">
-        <v>6.724528131648263</v>
+        <v>6.724528131648237</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>5.099017878523849</v>
+        <v>5.099017878520635</v>
       </c>
       <c r="I35" t="n">
-        <v>23.94338537308727</v>
+        <v>23.94338537308721</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>5.951571590283761</v>
+        <v>5.951571590284007</v>
       </c>
       <c r="L35" t="n">
-        <v>12.80721039317958</v>
+        <v>12.80721039317575</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1.220056913693688</v>
+        <v>1.220056913541201</v>
       </c>
       <c r="B36" t="n">
         <v>0</v>
@@ -1796,33 +1796,33 @@
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>7.117220573898448</v>
+        <v>7.11722057389845</v>
       </c>
       <c r="F36" t="n">
-        <v>6.80104312071458</v>
+        <v>6.801043120714596</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>5.167161373423991</v>
+        <v>5.167161373426362</v>
       </c>
       <c r="I36" t="n">
-        <v>23.60829563425076</v>
+        <v>23.60829563424215</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>6.034123164740941</v>
+        <v>6.034123164740935</v>
       </c>
       <c r="L36" t="n">
-        <v>12.62908260930837</v>
+        <v>12.6290826093082</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1.623790945734489</v>
+        <v>1.623790945521175</v>
       </c>
       <c r="B37" t="n">
         <v>0</v>
@@ -1834,33 +1834,33 @@
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>7.036525823518714</v>
+        <v>7.036525823518708</v>
       </c>
       <c r="F37" t="n">
-        <v>6.879412161042477</v>
+        <v>6.879412161042447</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>5.23436232746914</v>
+        <v>5.234362327483366</v>
       </c>
       <c r="I37" t="n">
-        <v>23.28719013934224</v>
+        <v>23.28719013922633</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>6.114834605629501</v>
+        <v>6.114834605629484</v>
       </c>
       <c r="L37" t="n">
-        <v>12.45969049902879</v>
+        <v>12.45969049902903</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>2.186736238782685</v>
+        <v>2.186736238823471</v>
       </c>
       <c r="B38" t="n">
         <v>0</v>
@@ -1872,33 +1872,33 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>6.955762599907265</v>
+        <v>6.955762599907269</v>
       </c>
       <c r="F38" t="n">
-        <v>6.959681763129194</v>
+        <v>6.959681763129237</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>5.300578531506626</v>
+        <v>5.300578531505893</v>
       </c>
       <c r="I38" t="n">
-        <v>22.97948170839178</v>
+        <v>22.97948170839738</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>6.18958445574463</v>
+        <v>6.189584455744591</v>
       </c>
       <c r="L38" t="n">
-        <v>12.30684554192779</v>
+        <v>12.30684554192704</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>2.782187956903099</v>
+        <v>2.782187956015926</v>
       </c>
       <c r="B39" t="n">
         <v>0</v>
@@ -1910,33 +1910,33 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>6.87495330071666</v>
+        <v>6.874953300716663</v>
       </c>
       <c r="F39" t="n">
-        <v>7.041898932091645</v>
+        <v>7.041898932091689</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>5.365770894385467</v>
+        <v>5.365770894360369</v>
       </c>
       <c r="I39" t="n">
-        <v>22.68460880172402</v>
+        <v>22.68460880226144</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>6.263269000128879</v>
+        <v>6.263269000125094</v>
       </c>
       <c r="L39" t="n">
-        <v>12.15983351180069</v>
+        <v>12.15983351180907</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>3.41023342062372</v>
+        <v>3.410233420704634</v>
       </c>
       <c r="B40" t="n">
         <v>0</v>
@@ -1948,33 +1948,33 @@
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>6.794121178772661</v>
+        <v>6.794121178772662</v>
       </c>
       <c r="F40" t="n">
-        <v>7.126111040903412</v>
+        <v>7.126111040903421</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>5.429903636838494</v>
+        <v>5.429903636832283</v>
       </c>
       <c r="I40" t="n">
-        <v>22.40203352792259</v>
+        <v>22.40203352797043</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>6.335855434439938</v>
+        <v>6.335855434439985</v>
       </c>
       <c r="L40" t="n">
-        <v>12.01843247146544</v>
+        <v>12.01843247146348</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4.070748177713827</v>
+        <v>4.070748177683578</v>
       </c>
       <c r="B41" t="n">
         <v>0</v>
@@ -1986,16 +1986,16 @@
         <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>6.713290391905609</v>
+        <v>6.713290391905606</v>
       </c>
       <c r="F41" t="n">
-        <v>7.212365680779611</v>
+        <v>7.212365680779768</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>5.492944454476768</v>
+        <v>5.492944454476767</v>
       </c>
       <c r="I41" t="n">
         <v>22.13123990479459</v>
@@ -2004,15 +2004,15 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>6.407313127950522</v>
+        <v>6.407313127951696</v>
       </c>
       <c r="L41" t="n">
-        <v>11.88242981402953</v>
+        <v>11.88242981403002</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>4.763381315069029</v>
+        <v>4.763381315114865</v>
       </c>
       <c r="B42" t="n">
         <v>0</v>
@@ -2024,33 +2024,33 @@
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>6.632486056001337</v>
+        <v>6.63248605600134</v>
       </c>
       <c r="F42" t="n">
-        <v>7.300710485690455</v>
+        <v>7.300710485690381</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>5.554864643466562</v>
+        <v>5.554864643466563</v>
       </c>
       <c r="I42" t="n">
-        <v>21.87173236185276</v>
+        <v>21.87173236185275</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>6.477613773440733</v>
+        <v>6.477613773438917</v>
       </c>
       <c r="L42" t="n">
-        <v>11.75162156798588</v>
+        <v>11.75162156798551</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>5.487543079383201</v>
+        <v>5.487543079605482</v>
       </c>
       <c r="B43" t="n">
         <v>0</v>
@@ -2065,30 +2065,30 @@
         <v>6.551734301450765</v>
       </c>
       <c r="F43" t="n">
-        <v>7.391192927639299</v>
+        <v>7.391192927639349</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>5.61563918274426</v>
+        <v>5.615639182744262</v>
       </c>
       <c r="I43" t="n">
-        <v>21.62303447646442</v>
+        <v>21.6230344764644</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>6.546731516664598</v>
+        <v>6.546731516644604</v>
       </c>
       <c r="L43" t="n">
-        <v>11.62581178152684</v>
+        <v>11.62581178154423</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>6.242395040274257</v>
+        <v>6.242395040237359</v>
       </c>
       <c r="B44" t="n">
         <v>0</v>
@@ -2100,33 +2100,33 @@
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>6.471062333178517</v>
+        <v>6.471062333178566</v>
       </c>
       <c r="F44" t="n">
-        <v>7.483860078972318</v>
+        <v>7.483860078971662</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>5.675246769240776</v>
+        <v>5.675246769240775</v>
       </c>
       <c r="I44" t="n">
-        <v>21.38468792566679</v>
+        <v>21.38468792566678</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>6.614643061932762</v>
+        <v>6.614643061934336</v>
       </c>
       <c r="L44" t="n">
-        <v>11.50481198234194</v>
+        <v>11.50481198234488</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>7.026842960152629</v>
+        <v>7.026842960284902</v>
       </c>
       <c r="B45" t="n">
         <v>0</v>
@@ -2138,16 +2138,16 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>6.390498494430958</v>
+        <v>6.390498494430956</v>
       </c>
       <c r="F45" t="n">
-        <v>7.578758337568981</v>
+        <v>7.578758337568939</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>5.733669804229781</v>
+        <v>5.733669804229779</v>
       </c>
       <c r="I45" t="n">
         <v>21.15625163373845</v>
@@ -2156,15 +2156,15 @@
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>6.681327751021728</v>
+        <v>6.681327750997908</v>
       </c>
       <c r="L45" t="n">
-        <v>11.38844070853454</v>
+        <v>11.38844070855768</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>7.839532457618419</v>
+        <v>7.839532457461945</v>
       </c>
       <c r="B46" t="n">
         <v>0</v>
@@ -2176,16 +2176,16 @@
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>6.310072334498395</v>
+        <v>6.31007233449836</v>
       </c>
       <c r="F46" t="n">
-        <v>7.675933110356115</v>
+        <v>7.675933110356645</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>5.79089433104874</v>
+        <v>5.790894331048739</v>
       </c>
       <c r="I46" t="n">
         <v>20.93730109162667</v>
@@ -2194,15 +2194,15 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>6.746767613261202</v>
+        <v>6.746767613246317</v>
       </c>
       <c r="L46" t="n">
-        <v>11.27652310557143</v>
+        <v>11.27652310559494</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>8.678847465526299</v>
+        <v>8.678847466207028</v>
       </c>
       <c r="B47" t="n">
         <v>0</v>
@@ -2214,33 +2214,33 @@
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>6.22981468054239</v>
+        <v>6.229814680542417</v>
       </c>
       <c r="F47" t="n">
-        <v>7.77542845008473</v>
+        <v>7.775428450084272</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>5.846909926361429</v>
+        <v>5.84690992636139</v>
       </c>
       <c r="I47" t="n">
-        <v>20.72742782215026</v>
+        <v>20.72742782215037</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>6.810947385913788</v>
+        <v>6.810947385861487</v>
       </c>
       <c r="L47" t="n">
-        <v>11.16889058376146</v>
+        <v>11.16889058381805</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>-3.538937443682084</v>
+        <v>-3.538937443681989</v>
       </c>
       <c r="B48" t="n">
         <v>0</v>
@@ -2252,28 +2252,28 @@
         <v>0.1</v>
       </c>
       <c r="E48" t="n">
-        <v>9.489621785789449</v>
+        <v>9.489621785789451</v>
       </c>
       <c r="F48" t="n">
-        <v>5.095529895621963</v>
+        <v>5.095529895621962</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>2.697430303624302</v>
+        <v>2.697430126586939</v>
       </c>
       <c r="I48" t="n">
-        <v>50.09930096397862</v>
+        <v>50.09929523907</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>3.092067073281464</v>
+        <v>3.092067197337133</v>
       </c>
       <c r="L48" t="n">
-        <v>25.25641123572337</v>
+        <v>25.25641030724787</v>
       </c>
     </row>
     <row r="49">
@@ -2293,30 +2293,30 @@
         <v>9.334823541325351</v>
       </c>
       <c r="F49" t="n">
-        <v>5.180257545197659</v>
+        <v>5.18025754519766</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>2.697430405444766</v>
+        <v>2.697430397701317</v>
       </c>
       <c r="I49" t="n">
-        <v>50.09930403406669</v>
+        <v>50.09930382112732</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
       </c>
       <c r="K49" t="n">
-        <v>3.09206716885968</v>
+        <v>3.09206729904317</v>
       </c>
       <c r="L49" t="n">
-        <v>25.25641047059553</v>
+        <v>25.25640955378933</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>-10.4495882656387</v>
+        <v>-10.44958826563855</v>
       </c>
       <c r="B50" t="n">
         <v>0</v>
@@ -2337,24 +2337,24 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>2.697430408004275</v>
+        <v>2.697430403631818</v>
       </c>
       <c r="I50" t="n">
-        <v>50.09930410377088</v>
+        <v>50.09930398475608</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>3.09206707396437</v>
+        <v>3.092067333040089</v>
       </c>
       <c r="L50" t="n">
-        <v>25.25641123187271</v>
+        <v>25.25640925531289</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>-13.82660796280592</v>
+        <v>-13.82660796280627</v>
       </c>
       <c r="B51" t="n">
         <v>0</v>
@@ -2366,33 +2366,33 @@
         <v>0.4</v>
       </c>
       <c r="E51" t="n">
-        <v>9.111589061977844</v>
+        <v>9.111589061977837</v>
       </c>
       <c r="F51" t="n">
-        <v>5.307534045233507</v>
+        <v>5.307534045233512</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>2.697430287309031</v>
+        <v>2.697430393490434</v>
       </c>
       <c r="I51" t="n">
-        <v>50.09930053925707</v>
+        <v>50.09930370514866</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>3.092067364570417</v>
+        <v>3.092067092660014</v>
       </c>
       <c r="L51" t="n">
-        <v>25.25640899724515</v>
+        <v>25.25641112531996</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>-30.14449406562217</v>
+        <v>-30.144494065624</v>
       </c>
       <c r="B52" t="n">
         <v>0</v>
@@ -2404,33 +2404,33 @@
         <v>0.9</v>
       </c>
       <c r="E52" t="n">
-        <v>8.771892049491537</v>
+        <v>8.771892049491504</v>
       </c>
       <c r="F52" t="n">
-        <v>5.513696461027553</v>
+        <v>5.513696461027649</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>2.697430374105616</v>
+        <v>2.697430306331713</v>
       </c>
       <c r="I52" t="n">
-        <v>50.09930313708208</v>
+        <v>50.0993010591862</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>3.092067061509431</v>
+        <v>3.092067080735457</v>
       </c>
       <c r="L52" t="n">
-        <v>25.25641130165692</v>
+        <v>25.25641119353691</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>2.102152324627045</v>
+        <v>2.102152324628775</v>
       </c>
       <c r="B53" t="n">
         <v>0</v>
@@ -2442,33 +2442,33 @@
         <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>9.699347069291402</v>
+        <v>9.699347069291424</v>
       </c>
       <c r="F53" t="n">
-        <v>4.985069224042757</v>
+        <v>4.985069224042792</v>
       </c>
       <c r="G53" t="n">
         <v>0.1</v>
       </c>
       <c r="H53" t="n">
-        <v>2.683989998574897</v>
+        <v>2.683989998574929</v>
       </c>
       <c r="I53" t="n">
-        <v>50.44368285083736</v>
+        <v>50.44368285083699</v>
       </c>
       <c r="J53" t="n">
         <v>0.1082177012392873</v>
       </c>
       <c r="K53" t="n">
-        <v>3.070883992165573</v>
+        <v>3.070883992165514</v>
       </c>
       <c r="L53" t="n">
-        <v>25.44301119189033</v>
+        <v>25.4430111918928</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>3.839251524594191</v>
+        <v>3.839251524612708</v>
       </c>
       <c r="B54" t="n">
         <v>0</v>
@@ -2483,30 +2483,30 @@
         <v>9.69934706929139</v>
       </c>
       <c r="F54" t="n">
-        <v>4.98506922404277</v>
+        <v>4.985069224042768</v>
       </c>
       <c r="G54" t="n">
         <v>0.2</v>
       </c>
       <c r="H54" t="n">
-        <v>2.672349906452419</v>
+        <v>2.672349906452221</v>
       </c>
       <c r="I54" t="n">
-        <v>50.74679737773776</v>
+        <v>50.74679737773828</v>
       </c>
       <c r="J54" t="n">
         <v>0.1861872028258322</v>
       </c>
       <c r="K54" t="n">
-        <v>3.056952118327394</v>
+        <v>3.056952118327383</v>
       </c>
       <c r="L54" t="n">
-        <v>25.56730559354525</v>
+        <v>25.56730559354667</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>5.484213403585476</v>
+        <v>5.484213403597066</v>
       </c>
       <c r="B55" t="n">
         <v>0</v>
@@ -2518,33 +2518,33 @@
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>9.699347069291393</v>
+        <v>9.699347069291395</v>
       </c>
       <c r="F55" t="n">
-        <v>4.985069224042768</v>
+        <v>4.985069224042769</v>
       </c>
       <c r="G55" t="n">
         <v>0.3</v>
       </c>
       <c r="H55" t="n">
-        <v>2.662052797422557</v>
+        <v>2.662052797422408</v>
       </c>
       <c r="I55" t="n">
-        <v>51.01881471155225</v>
+        <v>51.01881471155315</v>
       </c>
       <c r="J55" t="n">
         <v>0.2724584114361717</v>
       </c>
       <c r="K55" t="n">
-        <v>3.042562690630358</v>
+        <v>3.042562690630355</v>
       </c>
       <c r="L55" t="n">
-        <v>25.69701456619961</v>
+        <v>25.69701456619964</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>7.078163436590854</v>
+        <v>7.078163436514869</v>
       </c>
       <c r="B56" t="n">
         <v>0</v>
@@ -2556,33 +2556,33 @@
         <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>9.699347069291413</v>
+        <v>9.699347069291395</v>
       </c>
       <c r="F56" t="n">
-        <v>4.985069224042746</v>
+        <v>4.985069224042767</v>
       </c>
       <c r="G56" t="n">
         <v>0.4</v>
       </c>
       <c r="H56" t="n">
-        <v>2.652798813905597</v>
+        <v>2.652798813906231</v>
       </c>
       <c r="I56" t="n">
-        <v>51.26646119328322</v>
+        <v>51.26646119326673</v>
       </c>
       <c r="J56" t="n">
         <v>0.3709916581317118</v>
       </c>
       <c r="K56" t="n">
-        <v>3.027211975723692</v>
+        <v>3.027211975723695</v>
       </c>
       <c r="L56" t="n">
-        <v>25.83690649497285</v>
+        <v>25.83690649497283</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>14.09452555419575</v>
+        <v>14.09452555419547</v>
       </c>
       <c r="B57" t="n">
         <v>0</v>
@@ -2594,25 +2594,25 @@
         <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>9.699347069291418</v>
+        <v>9.699347069291392</v>
       </c>
       <c r="F57" t="n">
-        <v>4.985069224042745</v>
+        <v>4.985069224042769</v>
       </c>
       <c r="G57" t="n">
         <v>0.9</v>
       </c>
       <c r="H57" t="n">
-        <v>2.616554302275603</v>
+        <v>2.616554302275604</v>
       </c>
       <c r="I57" t="n">
-        <v>52.26686362450164</v>
+        <v>52.2668636245016</v>
       </c>
       <c r="J57" t="n">
         <v>0.9187962143520164</v>
       </c>
       <c r="K57" t="n">
-        <v>2.955899517665744</v>
+        <v>2.955899517665743</v>
       </c>
       <c r="L57" t="n">
         <v>26.50814840086409</v>
@@ -2620,7 +2620,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>2.388112351066671</v>
+        <v>2.388112351156182</v>
       </c>
       <c r="B58" t="n">
         <v>0</v>
@@ -2632,33 +2632,33 @@
         <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>9.699347069291413</v>
+        <v>9.699347069291422</v>
       </c>
       <c r="F58" t="n">
-        <v>4.985069224042779</v>
+        <v>4.985069224042783</v>
       </c>
       <c r="G58" t="n">
         <v>0.1247653346366633</v>
       </c>
       <c r="H58" t="n">
-        <v>2.680960870595422</v>
+        <v>2.680960870590401</v>
       </c>
       <c r="I58" t="n">
-        <v>50.52212255324282</v>
+        <v>50.52212255331549</v>
       </c>
       <c r="J58" t="n">
         <v>0.1</v>
       </c>
       <c r="K58" t="n">
-        <v>3.072411329380366</v>
+        <v>3.072411329380817</v>
       </c>
       <c r="L58" t="n">
-        <v>25.42946125386938</v>
+        <v>25.42946125384874</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>3.993545822174557</v>
+        <v>3.993545822059574</v>
       </c>
       <c r="B59" t="n">
         <v>0</v>
@@ -2670,16 +2670,16 @@
         <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>9.699347069291406</v>
+        <v>9.699347069291415</v>
       </c>
       <c r="F59" t="n">
-        <v>4.985069224042771</v>
+        <v>4.985069224042745</v>
       </c>
       <c r="G59" t="n">
         <v>0.2063981465460308</v>
       </c>
       <c r="H59" t="n">
-        <v>2.671654675914092</v>
+        <v>2.671654675914093</v>
       </c>
       <c r="I59" t="n">
         <v>50.76504750905971</v>
@@ -2688,15 +2688,15 @@
         <v>0.2</v>
       </c>
       <c r="K59" t="n">
-        <v>3.054581008433848</v>
+        <v>3.054581008435064</v>
       </c>
       <c r="L59" t="n">
-        <v>25.58858546719811</v>
+        <v>25.58858546705819</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>5.782095715150174</v>
+        <v>5.782095715022011</v>
       </c>
       <c r="B60" t="n">
         <v>0</v>
@@ -2711,30 +2711,30 @@
         <v>9.699347069291395</v>
       </c>
       <c r="F60" t="n">
-        <v>4.985069224042769</v>
+        <v>4.985069224042764</v>
       </c>
       <c r="G60" t="n">
         <v>0.3137697936590399</v>
       </c>
       <c r="H60" t="n">
-        <v>2.660722059192307</v>
+        <v>2.660722059192303</v>
       </c>
       <c r="I60" t="n">
-        <v>51.05423924417278</v>
+        <v>51.05423924417285</v>
       </c>
       <c r="J60" t="n">
         <v>0.3</v>
       </c>
       <c r="K60" t="n">
-        <v>3.038164646011364</v>
+        <v>3.038164646143399</v>
       </c>
       <c r="L60" t="n">
-        <v>25.73693289736029</v>
+        <v>25.73693290014568</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>7.248230992216799</v>
+        <v>7.248230992216659</v>
       </c>
       <c r="B61" t="n">
         <v>0</v>
@@ -2746,33 +2746,33 @@
         <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>9.699347069291408</v>
+        <v>9.699347069291395</v>
       </c>
       <c r="F61" t="n">
-        <v>4.985069224042771</v>
+        <v>4.98506922404277</v>
       </c>
       <c r="G61" t="n">
         <v>0.4026174994879254</v>
       </c>
       <c r="H61" t="n">
-        <v>2.652568566175737</v>
+        <v>2.652568566175738</v>
       </c>
       <c r="I61" t="n">
-        <v>51.27266195917268</v>
+        <v>51.27266195917266</v>
       </c>
       <c r="J61" t="n">
         <v>0.4</v>
       </c>
       <c r="K61" t="n">
-        <v>3.022883063824818</v>
+        <v>3.022883063824821</v>
       </c>
       <c r="L61" t="n">
-        <v>25.87664304552224</v>
+        <v>25.87664304552222</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>14.22767596066131</v>
+        <v>14.2276759606621</v>
       </c>
       <c r="B62" t="n">
         <v>0</v>
@@ -2784,33 +2784,33 @@
         <v>0</v>
       </c>
       <c r="E62" t="n">
-        <v>9.699347069291395</v>
+        <v>9.699347069291415</v>
       </c>
       <c r="F62" t="n">
-        <v>4.985069224042768</v>
+        <v>4.98506922404278</v>
       </c>
       <c r="G62" t="n">
         <v>0.9261043454272662</v>
       </c>
       <c r="H62" t="n">
-        <v>2.614983040688908</v>
+        <v>2.614983040688909</v>
       </c>
       <c r="I62" t="n">
-        <v>52.31137641976962</v>
+        <v>52.31137641976959</v>
       </c>
       <c r="J62" t="n">
         <v>0.9</v>
       </c>
       <c r="K62" t="n">
-        <v>2.958056868950862</v>
+        <v>2.958056868950858</v>
       </c>
       <c r="L62" t="n">
-        <v>26.48730884250889</v>
+        <v>26.48730884250892</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>-3.556607353125177</v>
+        <v>-3.556607353125074</v>
       </c>
       <c r="B63" t="n">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>0.1</v>
       </c>
       <c r="E63" t="n">
-        <v>8.419262476514666</v>
+        <v>8.419262476514668</v>
       </c>
       <c r="F63" t="n">
         <v>5.745391646600253</v>
@@ -2831,24 +2831,24 @@
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>3.743371491908506</v>
+        <v>3.743371734523987</v>
       </c>
       <c r="I63" t="n">
-        <v>33.55964653086292</v>
+        <v>33.55964318988732</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>4.395752719775719</v>
+        <v>4.395752719922317</v>
       </c>
       <c r="L63" t="n">
-        <v>17.46534079526109</v>
+        <v>17.46534079469805</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>-6.994453390141751</v>
+        <v>-6.99445339015288</v>
       </c>
       <c r="B64" t="n">
         <v>0</v>
@@ -2869,19 +2869,19 @@
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>3.743371856014079</v>
+        <v>3.743371856454088</v>
       </c>
       <c r="I64" t="n">
-        <v>33.55964144845556</v>
+        <v>33.55964144214902</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
       </c>
       <c r="K64" t="n">
-        <v>4.395752719914819</v>
+        <v>4.395752719922316</v>
       </c>
       <c r="L64" t="n">
-        <v>17.46534079473399</v>
+        <v>17.46534079469799</v>
       </c>
     </row>
     <row r="65">
@@ -2898,28 +2898,28 @@
         <v>0.3</v>
       </c>
       <c r="E65" t="n">
-        <v>8.162141933309721</v>
+        <v>8.162141933309719</v>
       </c>
       <c r="F65" t="n">
-        <v>5.927019035346338</v>
+        <v>5.92701903534634</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>3.743371434397131</v>
+        <v>3.743371836479491</v>
       </c>
       <c r="I65" t="n">
-        <v>33.55964715510039</v>
+        <v>33.55964173433919</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>4.395752719728842</v>
+        <v>4.395752719719552</v>
       </c>
       <c r="L65" t="n">
-        <v>17.46534079538619</v>
+        <v>17.46534079540978</v>
       </c>
     </row>
     <row r="66">
@@ -2936,28 +2936,28 @@
         <v>0.4</v>
       </c>
       <c r="E66" t="n">
-        <v>8.06740143910546</v>
+        <v>8.067401439105463</v>
       </c>
       <c r="F66" t="n">
-        <v>5.996877480197115</v>
+        <v>5.996877480197112</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
       </c>
       <c r="H66" t="n">
-        <v>3.743371856281114</v>
+        <v>3.743371736835742</v>
       </c>
       <c r="I66" t="n">
-        <v>33.55964144458471</v>
+        <v>33.55964316336497</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>4.395752719768211</v>
+        <v>4.395752719895895</v>
       </c>
       <c r="L66" t="n">
-        <v>17.46534079528188</v>
+        <v>17.46534079480371</v>
       </c>
     </row>
     <row r="67">
@@ -2974,28 +2974,28 @@
         <v>0.9</v>
       </c>
       <c r="E67" t="n">
-        <v>7.744056430685746</v>
+        <v>7.744056430685744</v>
       </c>
       <c r="F67" t="n">
-        <v>6.248247945552081</v>
+        <v>6.248247945552082</v>
       </c>
       <c r="G67" t="n">
         <v>0</v>
       </c>
       <c r="H67" t="n">
-        <v>3.743371856410349</v>
+        <v>3.743371473491525</v>
       </c>
       <c r="I67" t="n">
-        <v>33.5596414427964</v>
+        <v>33.55964673309816</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
       </c>
       <c r="K67" t="n">
-        <v>4.395752719920004</v>
+        <v>4.395752719607122</v>
       </c>
       <c r="L67" t="n">
-        <v>17.46534079471174</v>
+        <v>17.46534079591096</v>
       </c>
     </row>
     <row r="68">
@@ -3012,16 +3012,16 @@
         <v>0</v>
       </c>
       <c r="E68" t="n">
-        <v>8.61255600312302</v>
+        <v>8.612556003123018</v>
       </c>
       <c r="F68" t="n">
-        <v>5.616027178402859</v>
+        <v>5.616027178402819</v>
       </c>
       <c r="G68" t="n">
         <v>0.1</v>
       </c>
       <c r="H68" t="n">
-        <v>3.61464487639092</v>
+        <v>3.614644876390921</v>
       </c>
       <c r="I68" t="n">
         <v>34.92415151190161</v>
@@ -3038,7 +3038,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>33.72091318648222</v>
+        <v>33.7209131864819</v>
       </c>
       <c r="B69" t="n">
         <v>0</v>
@@ -3050,16 +3050,16 @@
         <v>0</v>
       </c>
       <c r="E69" t="n">
-        <v>8.612556003123018</v>
+        <v>8.61255600312302</v>
       </c>
       <c r="F69" t="n">
-        <v>5.61602717840287</v>
+        <v>5.616027178402838</v>
       </c>
       <c r="G69" t="n">
         <v>0.2</v>
       </c>
       <c r="H69" t="n">
-        <v>3.521833028281219</v>
+        <v>3.521833028281218</v>
       </c>
       <c r="I69" t="n">
         <v>35.98536345410113</v>
@@ -3068,10 +3068,10 @@
         <v>0.1861872028258322</v>
       </c>
       <c r="K69" t="n">
-        <v>4.049546550063069</v>
+        <v>4.04954655006307</v>
       </c>
       <c r="L69" t="n">
-        <v>19.01329900288214</v>
+        <v>19.01329900288213</v>
       </c>
     </row>
     <row r="70">
@@ -3088,16 +3088,16 @@
         <v>0</v>
       </c>
       <c r="E70" t="n">
-        <v>8.612556003123023</v>
+        <v>8.61255600312302</v>
       </c>
       <c r="F70" t="n">
-        <v>5.616027178402855</v>
+        <v>5.616027178402846</v>
       </c>
       <c r="G70" t="n">
         <v>0.3</v>
       </c>
       <c r="H70" t="n">
-        <v>3.450971586571708</v>
+        <v>3.450971586571707</v>
       </c>
       <c r="I70" t="n">
         <v>36.84438848520298</v>
@@ -3106,15 +3106,15 @@
         <v>0.2724584114361717</v>
       </c>
       <c r="K70" t="n">
-        <v>3.96087944603085</v>
+        <v>3.960879446030854</v>
       </c>
       <c r="L70" t="n">
-        <v>19.45586233971915</v>
+        <v>19.45586233971913</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>58.33905675691551</v>
+        <v>58.33905676017069</v>
       </c>
       <c r="B71" t="n">
         <v>0</v>
@@ -3126,33 +3126,33 @@
         <v>0</v>
       </c>
       <c r="E71" t="n">
-        <v>8.612556003123021</v>
+        <v>8.612556003123016</v>
       </c>
       <c r="F71" t="n">
-        <v>5.616027178402868</v>
+        <v>5.616027178402865</v>
       </c>
       <c r="G71" t="n">
         <v>0.4</v>
       </c>
       <c r="H71" t="n">
-        <v>3.394708122773546</v>
+        <v>3.3947081227438</v>
       </c>
       <c r="I71" t="n">
-        <v>37.55929838657981</v>
+        <v>37.55929838661633</v>
       </c>
       <c r="J71" t="n">
         <v>0.3709916581317118</v>
       </c>
       <c r="K71" t="n">
-        <v>3.885472523752267</v>
+        <v>3.885472523752266</v>
       </c>
       <c r="L71" t="n">
-        <v>19.84914493013566</v>
+        <v>19.84914493013567</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>101.6044903464519</v>
+        <v>101.6044903464645</v>
       </c>
       <c r="B72" t="n">
         <v>0</v>
@@ -3167,22 +3167,22 @@
         <v>8.61255600312302</v>
       </c>
       <c r="F72" t="n">
-        <v>5.616027178402857</v>
+        <v>5.616027178402861</v>
       </c>
       <c r="G72" t="n">
         <v>0.9</v>
       </c>
       <c r="H72" t="n">
-        <v>3.223645099627039</v>
+        <v>3.223645099626946</v>
       </c>
       <c r="I72" t="n">
-        <v>39.93586483587215</v>
+        <v>39.93586483587221</v>
       </c>
       <c r="J72" t="n">
         <v>0.9187962143520164</v>
       </c>
       <c r="K72" t="n">
-        <v>3.666551565360047</v>
+        <v>3.666551565360048</v>
       </c>
       <c r="L72" t="n">
         <v>21.08903337881345</v>
@@ -3190,7 +3190,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>21.37829750524171</v>
+        <v>21.37829750522033</v>
       </c>
       <c r="B73" t="n">
         <v>0</v>
@@ -3202,33 +3202,33 @@
         <v>0</v>
       </c>
       <c r="E73" t="n">
-        <v>8.612556003123018</v>
+        <v>8.61255600312302</v>
       </c>
       <c r="F73" t="n">
-        <v>5.61602717840287</v>
+        <v>5.616027178402855</v>
       </c>
       <c r="G73" t="n">
         <v>0.1247653346366633</v>
       </c>
       <c r="H73" t="n">
-        <v>3.589027608060948</v>
+        <v>3.589027608061252</v>
       </c>
       <c r="I73" t="n">
-        <v>35.2102006432139</v>
+        <v>35.21020064321461</v>
       </c>
       <c r="J73" t="n">
         <v>0.1</v>
       </c>
       <c r="K73" t="n">
-        <v>4.173296784901265</v>
+        <v>4.173296784901269</v>
       </c>
       <c r="L73" t="n">
-        <v>18.42886757135937</v>
+        <v>18.42886757135935</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>35.00167089836352</v>
+        <v>35.00167089836386</v>
       </c>
       <c r="B74" t="n">
         <v>0</v>
@@ -3243,25 +3243,25 @@
         <v>8.612556003123021</v>
       </c>
       <c r="F74" t="n">
-        <v>5.616027178402834</v>
+        <v>5.61602717840285</v>
       </c>
       <c r="G74" t="n">
         <v>0.2063981465460308</v>
       </c>
       <c r="H74" t="n">
-        <v>3.516742338019175</v>
+        <v>3.516742338019172</v>
       </c>
       <c r="I74" t="n">
-        <v>36.04561280808695</v>
+        <v>36.045612808087</v>
       </c>
       <c r="J74" t="n">
         <v>0.2</v>
       </c>
       <c r="K74" t="n">
-        <v>4.033441996411134</v>
+        <v>4.033441996411131</v>
       </c>
       <c r="L74" t="n">
-        <v>19.09214830533379</v>
+        <v>19.0921483053338</v>
       </c>
     </row>
     <row r="75">
@@ -3281,30 +3281,30 @@
         <v>8.61255600312302</v>
       </c>
       <c r="F75" t="n">
-        <v>5.616027178402858</v>
+        <v>5.616027178402865</v>
       </c>
       <c r="G75" t="n">
         <v>0.3137697936590399</v>
       </c>
       <c r="H75" t="n">
-        <v>3.442478302831986</v>
+        <v>3.442478302831989</v>
       </c>
       <c r="I75" t="n">
-        <v>36.95038383171704</v>
+        <v>36.950383831717</v>
       </c>
       <c r="J75" t="n">
         <v>0.3</v>
       </c>
       <c r="K75" t="n">
-        <v>3.937554987460157</v>
+        <v>3.937554987460162</v>
       </c>
       <c r="L75" t="n">
-        <v>19.57579927509693</v>
+        <v>19.5757992750969</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>59.45245776562128</v>
+        <v>59.45245776565447</v>
       </c>
       <c r="B76" t="n">
         <v>0</v>
@@ -3316,33 +3316,33 @@
         <v>0</v>
       </c>
       <c r="E76" t="n">
-        <v>8.612556003123021</v>
+        <v>8.61255600312302</v>
       </c>
       <c r="F76" t="n">
-        <v>5.616027178402834</v>
+        <v>5.616027178402838</v>
       </c>
       <c r="G76" t="n">
         <v>0.4026174994879254</v>
       </c>
       <c r="H76" t="n">
-        <v>3.393387678295042</v>
+        <v>3.393387678294769</v>
       </c>
       <c r="I76" t="n">
-        <v>37.57644467614871</v>
+        <v>37.57644467614968</v>
       </c>
       <c r="J76" t="n">
         <v>0.4</v>
       </c>
       <c r="K76" t="n">
-        <v>3.866911644169634</v>
+        <v>3.86691164416963</v>
       </c>
       <c r="L76" t="n">
-        <v>19.94845421713874</v>
+        <v>19.94845421713876</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>102.638124663748</v>
+        <v>102.6381246652596</v>
       </c>
       <c r="B77" t="n">
         <v>0</v>
@@ -3357,16 +3357,16 @@
         <v>8.61255600312302</v>
       </c>
       <c r="F77" t="n">
-        <v>5.616027178402859</v>
+        <v>5.616027178402845</v>
       </c>
       <c r="G77" t="n">
         <v>0.9261043454272662</v>
       </c>
       <c r="H77" t="n">
-        <v>3.21758285243637</v>
+        <v>3.217582852426232</v>
       </c>
       <c r="I77" t="n">
-        <v>40.02630051774122</v>
+        <v>40.02630051775188</v>
       </c>
       <c r="J77" t="n">
         <v>0.9</v>
@@ -3392,28 +3392,28 @@
         <v>0.1</v>
       </c>
       <c r="E78" t="n">
-        <v>7.658962145149544</v>
+        <v>7.658962145149542</v>
       </c>
       <c r="F78" t="n">
-        <v>6.317949772334973</v>
+        <v>6.317949772334975</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
       </c>
       <c r="H78" t="n">
-        <v>4.509158846995403</v>
+        <v>4.509158846995454</v>
       </c>
       <c r="I78" t="n">
-        <v>27.31758801122518</v>
+        <v>27.31758801122306</v>
       </c>
       <c r="J78" t="n">
         <v>0</v>
       </c>
       <c r="K78" t="n">
-        <v>5.272990572693508</v>
+        <v>5.272990572691759</v>
       </c>
       <c r="L78" t="n">
-        <v>14.48923362419594</v>
+        <v>14.48923362420006</v>
       </c>
     </row>
     <row r="79">
@@ -3430,28 +3430,28 @@
         <v>0.2</v>
       </c>
       <c r="E79" t="n">
-        <v>7.525051081621916</v>
+        <v>7.525051081621912</v>
       </c>
       <c r="F79" t="n">
-        <v>6.430850327703494</v>
+        <v>6.430850327703497</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>4.509158846995449</v>
+        <v>4.509158846318763</v>
       </c>
       <c r="I79" t="n">
-        <v>27.31758801122301</v>
+        <v>27.3175880173613</v>
       </c>
       <c r="J79" t="n">
         <v>0</v>
       </c>
       <c r="K79" t="n">
-        <v>5.272990572696991</v>
+        <v>5.272990572696992</v>
       </c>
       <c r="L79" t="n">
-        <v>14.48923362418054</v>
+        <v>14.48923362418111</v>
       </c>
     </row>
     <row r="80">
@@ -3468,28 +3468,28 @@
         <v>0.3</v>
       </c>
       <c r="E80" t="n">
-        <v>7.417853743579847</v>
+        <v>7.417853743579846</v>
       </c>
       <c r="F80" t="n">
-        <v>6.524185059903331</v>
+        <v>6.524185059903333</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>4.509158846995455</v>
+        <v>4.509158846992159</v>
       </c>
       <c r="I80" t="n">
-        <v>27.3175880112232</v>
+        <v>27.31758801128926</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
       </c>
       <c r="K80" t="n">
-        <v>5.272990572696822</v>
+        <v>5.272990572696991</v>
       </c>
       <c r="L80" t="n">
-        <v>14.48923362418303</v>
+        <v>14.48923362418046</v>
       </c>
     </row>
     <row r="81">
@@ -3506,28 +3506,28 @@
         <v>0.4</v>
       </c>
       <c r="E81" t="n">
-        <v>7.328660955698762</v>
+        <v>7.328660955698759</v>
       </c>
       <c r="F81" t="n">
-        <v>6.603938387878665</v>
+        <v>6.603938387878668</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>4.509158846908393</v>
+        <v>4.509158846994992</v>
       </c>
       <c r="I81" t="n">
-        <v>27.31758801200958</v>
+        <v>27.31758801123436</v>
       </c>
       <c r="J81" t="n">
         <v>0</v>
       </c>
       <c r="K81" t="n">
-        <v>5.27299057269699</v>
+        <v>5.272990572696993</v>
       </c>
       <c r="L81" t="n">
-        <v>14.48923362418117</v>
+        <v>14.48923362418114</v>
       </c>
     </row>
     <row r="82">
@@ -3544,7 +3544,7 @@
         <v>0.9</v>
       </c>
       <c r="E82" t="n">
-        <v>7.02759939761558</v>
+        <v>7.027599397615582</v>
       </c>
       <c r="F82" t="n">
         <v>6.888192676121482</v>
@@ -3553,24 +3553,24 @@
         <v>0</v>
       </c>
       <c r="H82" t="n">
-        <v>4.509158846995449</v>
+        <v>4.50915884699542</v>
       </c>
       <c r="I82" t="n">
-        <v>27.3175880112231</v>
+        <v>27.31758801122416</v>
       </c>
       <c r="J82" t="n">
         <v>0</v>
       </c>
       <c r="K82" t="n">
-        <v>5.272990572696989</v>
+        <v>5.272990572696103</v>
       </c>
       <c r="L82" t="n">
-        <v>14.48923362418039</v>
+        <v>14.48923362418668</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>24.35280591724352</v>
+        <v>24.35280591724307</v>
       </c>
       <c r="B83" t="n">
         <v>0</v>
@@ -3582,19 +3582,19 @@
         <v>0</v>
       </c>
       <c r="E83" t="n">
-        <v>7.837064168615012</v>
+        <v>7.837064168615006</v>
       </c>
       <c r="F83" t="n">
-        <v>6.173805682149561</v>
+        <v>6.173805682149524</v>
       </c>
       <c r="G83" t="n">
         <v>0.1</v>
       </c>
       <c r="H83" t="n">
-        <v>4.335524995031109</v>
+        <v>4.335524995031112</v>
       </c>
       <c r="I83" t="n">
-        <v>28.50932177756017</v>
+        <v>28.50932177756015</v>
       </c>
       <c r="J83" t="n">
         <v>0.1082177012392873</v>
@@ -3620,10 +3620,10 @@
         <v>0</v>
       </c>
       <c r="E84" t="n">
-        <v>7.837064168615007</v>
+        <v>7.837064168615009</v>
       </c>
       <c r="F84" t="n">
-        <v>6.173805682149554</v>
+        <v>6.173805682149539</v>
       </c>
       <c r="G84" t="n">
         <v>0.2</v>
@@ -3638,10 +3638,10 @@
         <v>0.1861872028258322</v>
       </c>
       <c r="K84" t="n">
-        <v>4.793578934046007</v>
+        <v>4.793578934046012</v>
       </c>
       <c r="L84" t="n">
-        <v>15.97516621938441</v>
+        <v>15.97516621938439</v>
       </c>
     </row>
     <row r="85">
@@ -3658,28 +3658,28 @@
         <v>0</v>
       </c>
       <c r="E85" t="n">
-        <v>7.837064168615009</v>
+        <v>7.837064168615006</v>
       </c>
       <c r="F85" t="n">
-        <v>6.173805682149569</v>
+        <v>6.17380568214955</v>
       </c>
       <c r="G85" t="n">
         <v>0.3</v>
       </c>
       <c r="H85" t="n">
-        <v>4.11246745646153</v>
+        <v>4.112467456461531</v>
       </c>
       <c r="I85" t="n">
-        <v>30.21129176485882</v>
+        <v>30.21129176485881</v>
       </c>
       <c r="J85" t="n">
         <v>0.2724584114361717</v>
       </c>
       <c r="K85" t="n">
-        <v>4.647643714064566</v>
+        <v>4.647643714064562</v>
       </c>
       <c r="L85" t="n">
-        <v>16.49087103004834</v>
+        <v>16.49087103004835</v>
       </c>
     </row>
     <row r="86">
@@ -3696,16 +3696,16 @@
         <v>0</v>
       </c>
       <c r="E86" t="n">
-        <v>7.837064168615007</v>
+        <v>7.837064168615004</v>
       </c>
       <c r="F86" t="n">
-        <v>6.173805682149557</v>
+        <v>6.173805682149561</v>
       </c>
       <c r="G86" t="n">
         <v>0.4</v>
       </c>
       <c r="H86" t="n">
-        <v>4.032194573316414</v>
+        <v>4.032194573316413</v>
       </c>
       <c r="I86" t="n">
         <v>30.87773509975563</v>
@@ -3714,7 +3714,7 @@
         <v>0.3709916581317118</v>
       </c>
       <c r="K86" t="n">
-        <v>4.513984366932661</v>
+        <v>4.513984366932663</v>
       </c>
       <c r="L86" t="n">
         <v>16.9937723594608</v>
@@ -3722,7 +3722,7 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>166.051787943253</v>
+        <v>166.0517879422206</v>
       </c>
       <c r="B87" t="n">
         <v>0</v>
@@ -3737,25 +3737,25 @@
         <v>7.837064168615006</v>
       </c>
       <c r="F87" t="n">
-        <v>6.173805682149553</v>
+        <v>6.173805682149551</v>
       </c>
       <c r="G87" t="n">
         <v>0.9</v>
       </c>
       <c r="H87" t="n">
-        <v>3.76654313947536</v>
+        <v>3.766543139479575</v>
       </c>
       <c r="I87" t="n">
-        <v>33.32612956193377</v>
+        <v>33.32612956190602</v>
       </c>
       <c r="J87" t="n">
         <v>0.9187962143520164</v>
       </c>
       <c r="K87" t="n">
-        <v>4.105149470269706</v>
+        <v>4.105149470269883</v>
       </c>
       <c r="L87" t="n">
-        <v>18.74609482972911</v>
+        <v>18.74609482972849</v>
       </c>
     </row>
     <row r="88">
@@ -3775,22 +3775,22 @@
         <v>7.837064168615006</v>
       </c>
       <c r="F88" t="n">
-        <v>6.173805682149554</v>
+        <v>6.173805682149535</v>
       </c>
       <c r="G88" t="n">
         <v>0.1247653346366633</v>
       </c>
       <c r="H88" t="n">
-        <v>4.301130354332845</v>
+        <v>4.30113035433284</v>
       </c>
       <c r="I88" t="n">
-        <v>28.75848174617386</v>
+        <v>28.7584817461739</v>
       </c>
       <c r="J88" t="n">
         <v>0.1</v>
       </c>
       <c r="K88" t="n">
-        <v>4.977885818595451</v>
+        <v>4.97788581859545</v>
       </c>
       <c r="L88" t="n">
         <v>15.36877144665517</v>
@@ -3798,7 +3798,7 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>46.1624987222564</v>
+        <v>46.16249872225677</v>
       </c>
       <c r="B89" t="n">
         <v>0</v>
@@ -3810,10 +3810,10 @@
         <v>0</v>
       </c>
       <c r="E89" t="n">
-        <v>7.837064168615007</v>
+        <v>7.837064168615009</v>
       </c>
       <c r="F89" t="n">
-        <v>6.173805682149556</v>
+        <v>6.17380568214955</v>
       </c>
       <c r="G89" t="n">
         <v>0.2063981465460308</v>
@@ -3828,15 +3828,15 @@
         <v>0.2</v>
       </c>
       <c r="K89" t="n">
-        <v>4.767998876531849</v>
+        <v>4.767998876531847</v>
       </c>
       <c r="L89" t="n">
-        <v>16.06318375226907</v>
+        <v>16.06318375226908</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>67.33349544284323</v>
+        <v>67.33349544284391</v>
       </c>
       <c r="B90" t="n">
         <v>0</v>
@@ -3851,30 +3851,30 @@
         <v>7.837064168615006</v>
       </c>
       <c r="F90" t="n">
-        <v>6.173805682149555</v>
+        <v>6.17380568214953</v>
       </c>
       <c r="G90" t="n">
         <v>0.3137697936590399</v>
       </c>
       <c r="H90" t="n">
-        <v>4.100520633784763</v>
+        <v>4.100520633784759</v>
       </c>
       <c r="I90" t="n">
-        <v>30.30853986447129</v>
+        <v>30.30853986447131</v>
       </c>
       <c r="J90" t="n">
         <v>0.3</v>
       </c>
       <c r="K90" t="n">
-        <v>4.607184891544382</v>
+        <v>4.607184891544377</v>
       </c>
       <c r="L90" t="n">
-        <v>16.63988212863547</v>
+        <v>16.63988212863548</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>85.06366876632356</v>
+        <v>85.0636687663243</v>
       </c>
       <c r="B91" t="n">
         <v>0</v>
@@ -3886,16 +3886,16 @@
         <v>0</v>
       </c>
       <c r="E91" t="n">
-        <v>7.837064168615009</v>
+        <v>7.837064168615007</v>
       </c>
       <c r="F91" t="n">
-        <v>6.173805682149575</v>
+        <v>6.173805682149577</v>
       </c>
       <c r="G91" t="n">
         <v>0.4026174994879254</v>
       </c>
       <c r="H91" t="n">
-        <v>4.0302758839185</v>
+        <v>4.030275883918499</v>
       </c>
       <c r="I91" t="n">
         <v>30.89404689015254</v>
@@ -3904,15 +3904,15 @@
         <v>0.4</v>
       </c>
       <c r="K91" t="n">
-        <v>4.479934196712301</v>
+        <v>4.479934196712302</v>
       </c>
       <c r="L91" t="n">
-        <v>17.12690822717056</v>
+        <v>17.12690822717055</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>167.8955230012027</v>
+        <v>167.8955230012453</v>
       </c>
       <c r="B92" t="n">
         <v>0</v>
@@ -3924,16 +3924,16 @@
         <v>0</v>
       </c>
       <c r="E92" t="n">
-        <v>7.837064168615006</v>
+        <v>7.837064168615009</v>
       </c>
       <c r="F92" t="n">
-        <v>6.17380568214956</v>
+        <v>6.173805682149546</v>
       </c>
       <c r="G92" t="n">
         <v>0.9261043454272662</v>
       </c>
       <c r="H92" t="n">
-        <v>3.756446993650571</v>
+        <v>3.756446993650572</v>
       </c>
       <c r="I92" t="n">
         <v>33.42744356830013</v>
@@ -3942,15 +3942,15 @@
         <v>0.9</v>
       </c>
       <c r="K92" t="n">
-        <v>4.113852220028178</v>
+        <v>4.113852220027621</v>
       </c>
       <c r="L92" t="n">
-        <v>18.70496455751945</v>
+        <v>18.70496455751894</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>-1.332170214856333</v>
+        <v>-1.332170215260652</v>
       </c>
       <c r="B93" t="n">
         <v>0</v>
@@ -3962,33 +3962,33 @@
         <v>0.1</v>
       </c>
       <c r="E93" t="n">
-        <v>6.881596036859924</v>
+        <v>6.881596036859921</v>
       </c>
       <c r="F93" t="n">
-        <v>7.035067073026367</v>
+        <v>7.035067073026371</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
       </c>
       <c r="H93" t="n">
-        <v>5.234362327473655</v>
+        <v>5.234362327483119</v>
       </c>
       <c r="I93" t="n">
-        <v>23.28719013922434</v>
+        <v>23.28719013923213</v>
       </c>
       <c r="J93" t="n">
         <v>0</v>
       </c>
       <c r="K93" t="n">
-        <v>6.114834605628894</v>
+        <v>6.114834605629476</v>
       </c>
       <c r="L93" t="n">
-        <v>12.4596904990298</v>
+        <v>12.45969049902896</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>-4.049495629276092</v>
+        <v>-4.049495629541639</v>
       </c>
       <c r="B94" t="n">
         <v>0</v>
@@ -4000,33 +4000,33 @@
         <v>0.2</v>
       </c>
       <c r="E94" t="n">
-        <v>6.766664235926041</v>
+        <v>6.766664235926038</v>
       </c>
       <c r="F94" t="n">
-        <v>7.155177451354788</v>
+        <v>7.155177451354792</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
       </c>
       <c r="H94" t="n">
-        <v>5.234362327461625</v>
+        <v>5.234362327483369</v>
       </c>
       <c r="I94" t="n">
-        <v>23.28719013941486</v>
+        <v>23.28719013922632</v>
       </c>
       <c r="J94" t="n">
         <v>0</v>
       </c>
       <c r="K94" t="n">
-        <v>6.114834605629452</v>
+        <v>6.114834605629451</v>
       </c>
       <c r="L94" t="n">
-        <v>12.45969049902895</v>
+        <v>12.45969049902891</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>-6.567710567906022</v>
+        <v>-6.567710567833331</v>
       </c>
       <c r="B95" t="n">
         <v>0</v>
@@ -4038,33 +4038,33 @@
         <v>0.3</v>
       </c>
       <c r="E95" t="n">
-        <v>6.676228233285356</v>
+        <v>6.676228233286731</v>
       </c>
       <c r="F95" t="n">
-        <v>7.25261875260166</v>
+        <v>7.252618752601803</v>
       </c>
       <c r="G95" t="n">
         <v>0</v>
       </c>
       <c r="H95" t="n">
-        <v>5.234362327483132</v>
+        <v>5.234362327482882</v>
       </c>
       <c r="I95" t="n">
-        <v>23.28719013923191</v>
+        <v>23.28719013923107</v>
       </c>
       <c r="J95" t="n">
         <v>0</v>
       </c>
       <c r="K95" t="n">
-        <v>6.114834605629493</v>
+        <v>6.114834605629484</v>
       </c>
       <c r="L95" t="n">
-        <v>12.45969049902883</v>
+        <v>12.45969049902886</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>-8.916920732880685</v>
+        <v>-8.916920733186998</v>
       </c>
       <c r="B96" t="n">
         <v>0</v>
@@ -4076,33 +4076,33 @@
         <v>0.4</v>
       </c>
       <c r="E96" t="n">
-        <v>6.602232654388004</v>
+        <v>6.602232654372989</v>
       </c>
       <c r="F96" t="n">
-        <v>7.334348027625421</v>
+        <v>7.334348027642058</v>
       </c>
       <c r="G96" t="n">
         <v>0</v>
       </c>
       <c r="H96" t="n">
-        <v>5.234362327483363</v>
+        <v>5.234362327480314</v>
       </c>
       <c r="I96" t="n">
-        <v>23.28719013922635</v>
+        <v>23.28719013923874</v>
       </c>
       <c r="J96" t="n">
         <v>0</v>
       </c>
       <c r="K96" t="n">
-        <v>6.114834605629477</v>
+        <v>6.114834605629428</v>
       </c>
       <c r="L96" t="n">
-        <v>12.45969049902877</v>
+        <v>12.45969049902893</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>-18.81803641841031</v>
+        <v>-18.81803641830559</v>
       </c>
       <c r="B97" t="n">
         <v>0</v>
@@ -4114,33 +4114,33 @@
         <v>0.9</v>
       </c>
       <c r="E97" t="n">
-        <v>6.361184206158711</v>
+        <v>6.361184206158725</v>
       </c>
       <c r="F97" t="n">
-        <v>7.613890141625032</v>
+        <v>7.61389014162499</v>
       </c>
       <c r="G97" t="n">
         <v>0</v>
       </c>
       <c r="H97" t="n">
-        <v>5.234362327483369</v>
+        <v>5.234362327481742</v>
       </c>
       <c r="I97" t="n">
-        <v>23.28719013922631</v>
+        <v>23.28719013923457</v>
       </c>
       <c r="J97" t="n">
         <v>0</v>
       </c>
       <c r="K97" t="n">
-        <v>6.114834605629372</v>
+        <v>6.114834605629454</v>
       </c>
       <c r="L97" t="n">
-        <v>12.45969049902921</v>
+        <v>12.45969049902894</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>26.3347781324592</v>
+        <v>26.3347781324589</v>
       </c>
       <c r="B98" t="n">
         <v>0</v>
@@ -4152,19 +4152,19 @@
         <v>0</v>
       </c>
       <c r="E98" t="n">
-        <v>7.03652582351871</v>
+        <v>7.036525823518705</v>
       </c>
       <c r="F98" t="n">
-        <v>6.879412161042484</v>
+        <v>6.87941216104238</v>
       </c>
       <c r="G98" t="n">
         <v>0.1</v>
       </c>
       <c r="H98" t="n">
-        <v>5.052738297533367</v>
+        <v>5.052738297533373</v>
       </c>
       <c r="I98" t="n">
-        <v>24.17662715341196</v>
+        <v>24.17662715341194</v>
       </c>
       <c r="J98" t="n">
         <v>0.1082177012392873</v>
@@ -4178,7 +4178,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>47.70273922685348</v>
+        <v>47.70273922685402</v>
       </c>
       <c r="B99" t="n">
         <v>0</v>
@@ -4190,33 +4190,33 @@
         <v>0</v>
       </c>
       <c r="E99" t="n">
-        <v>7.036525823518708</v>
+        <v>7.036525823518714</v>
       </c>
       <c r="F99" t="n">
-        <v>6.879412161042415</v>
+        <v>6.879412161042475</v>
       </c>
       <c r="G99" t="n">
         <v>0.2</v>
       </c>
       <c r="H99" t="n">
-        <v>4.910237968469839</v>
+        <v>4.910237968469831</v>
       </c>
       <c r="I99" t="n">
-        <v>24.92531420114916</v>
+        <v>24.92531420114917</v>
       </c>
       <c r="J99" t="n">
         <v>0.1861872028258322</v>
       </c>
       <c r="K99" t="n">
-        <v>5.569182817693889</v>
+        <v>5.569182817693894</v>
       </c>
       <c r="L99" t="n">
-        <v>13.70314677153785</v>
+        <v>13.70314677153784</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>69.5288724871215</v>
+        <v>69.52887248711305</v>
       </c>
       <c r="B100" t="n">
         <v>0</v>
@@ -4228,33 +4228,33 @@
         <v>0</v>
       </c>
       <c r="E100" t="n">
-        <v>7.036525823518708</v>
+        <v>7.036525823518712</v>
       </c>
       <c r="F100" t="n">
-        <v>6.879412161042429</v>
+        <v>6.879412161042444</v>
       </c>
       <c r="G100" t="n">
         <v>0.3</v>
       </c>
       <c r="H100" t="n">
-        <v>4.793680444460562</v>
+        <v>4.79368044446063</v>
       </c>
       <c r="I100" t="n">
-        <v>25.57445800156789</v>
+        <v>25.57445800156761</v>
       </c>
       <c r="J100" t="n">
         <v>0.2724584114361717</v>
       </c>
       <c r="K100" t="n">
-        <v>5.404204350756454</v>
+        <v>5.40420435075646</v>
       </c>
       <c r="L100" t="n">
-        <v>14.13002829260943</v>
+        <v>14.13002829260942</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>91.57591160279156</v>
+        <v>91.57591160279111</v>
       </c>
       <c r="B101" t="n">
         <v>0</v>
@@ -4266,10 +4266,10 @@
         <v>0</v>
       </c>
       <c r="E101" t="n">
-        <v>7.036525823518708</v>
+        <v>7.036525823518714</v>
       </c>
       <c r="F101" t="n">
-        <v>6.879412161042457</v>
+        <v>6.879412161042461</v>
       </c>
       <c r="G101" t="n">
         <v>0.4</v>
@@ -4284,15 +4284,15 @@
         <v>0.3709916581317118</v>
       </c>
       <c r="K101" t="n">
-        <v>5.250672918035875</v>
+        <v>5.250672918035882</v>
       </c>
       <c r="L101" t="n">
-        <v>14.55217543507358</v>
+        <v>14.55217543507356</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>195.769790155638</v>
+        <v>195.7697901556399</v>
       </c>
       <c r="B102" t="n">
         <v>0</v>
@@ -4304,33 +4304,33 @@
         <v>0</v>
       </c>
       <c r="E102" t="n">
-        <v>7.036525823518715</v>
+        <v>7.036525823518707</v>
       </c>
       <c r="F102" t="n">
-        <v>6.87941216104245</v>
+        <v>6.879412161042403</v>
       </c>
       <c r="G102" t="n">
         <v>0.9</v>
       </c>
       <c r="H102" t="n">
-        <v>4.389800427566256</v>
+        <v>4.38980042756626</v>
       </c>
       <c r="I102" t="n">
-        <v>28.12523679037499</v>
+        <v>28.12523679037497</v>
       </c>
       <c r="J102" t="n">
         <v>0.9187962143520164</v>
       </c>
       <c r="K102" t="n">
-        <v>4.713439010305852</v>
+        <v>4.713439010305819</v>
       </c>
       <c r="L102" t="n">
-        <v>16.25424305335352</v>
+        <v>16.25424305335354</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>28.98896336111186</v>
+        <v>28.98896336111157</v>
       </c>
       <c r="B103" t="n">
         <v>0</v>
@@ -4342,10 +4342,10 @@
         <v>0</v>
       </c>
       <c r="E103" t="n">
-        <v>7.036525823518705</v>
+        <v>7.036525823518709</v>
       </c>
       <c r="F103" t="n">
-        <v>6.879412161042408</v>
+        <v>6.879412161042465</v>
       </c>
       <c r="G103" t="n">
         <v>0.1247653346366633</v>
@@ -4354,21 +4354,21 @@
         <v>5.01422572594895</v>
       </c>
       <c r="I103" t="n">
-        <v>24.37434002473973</v>
+        <v>24.37434002473972</v>
       </c>
       <c r="J103" t="n">
         <v>0.1</v>
       </c>
       <c r="K103" t="n">
-        <v>5.778561248032205</v>
+        <v>5.778561248032207</v>
       </c>
       <c r="L103" t="n">
-        <v>13.19748050013088</v>
+        <v>13.19748050013087</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>49.86104721298723</v>
+        <v>49.86104721299763</v>
       </c>
       <c r="B104" t="n">
         <v>0</v>
@@ -4383,22 +4383,22 @@
         <v>7.036525823518712</v>
       </c>
       <c r="F104" t="n">
-        <v>6.879412161042455</v>
+        <v>6.879412161042437</v>
       </c>
       <c r="G104" t="n">
         <v>0.2063981465460308</v>
       </c>
       <c r="H104" t="n">
-        <v>4.902195711594073</v>
+        <v>4.902195711593977</v>
       </c>
       <c r="I104" t="n">
-        <v>24.96900398019909</v>
+        <v>24.96900398019946</v>
       </c>
       <c r="J104" t="n">
         <v>0.2</v>
       </c>
       <c r="K104" t="n">
-        <v>5.540289473033624</v>
+        <v>5.540289473033623</v>
       </c>
       <c r="L104" t="n">
         <v>13.77601630590739</v>
@@ -4406,7 +4406,7 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>73.82948992900793</v>
+        <v>73.82948992900836</v>
       </c>
       <c r="B105" t="n">
         <v>0</v>
@@ -4421,30 +4421,30 @@
         <v>7.036525823518715</v>
       </c>
       <c r="F105" t="n">
-        <v>6.879412161042474</v>
+        <v>6.879412161042478</v>
       </c>
       <c r="G105" t="n">
         <v>0.3137697936590399</v>
       </c>
       <c r="H105" t="n">
-        <v>4.779478728641965</v>
+        <v>4.77947872864197</v>
       </c>
       <c r="I105" t="n">
-        <v>25.65596181732004</v>
+        <v>25.65596181732001</v>
       </c>
       <c r="J105" t="n">
         <v>0.3</v>
       </c>
       <c r="K105" t="n">
-        <v>5.358158620144749</v>
+        <v>5.358158620144747</v>
       </c>
       <c r="L105" t="n">
-        <v>14.25401270430055</v>
+        <v>14.25401270430056</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>94.33705261420074</v>
+        <v>94.33705261420045</v>
       </c>
       <c r="B106" t="n">
         <v>0</v>
@@ -4456,33 +4456,33 @@
         <v>0</v>
       </c>
       <c r="E106" t="n">
-        <v>7.036525823518714</v>
+        <v>7.036525823518712</v>
       </c>
       <c r="F106" t="n">
-        <v>6.879412161042461</v>
+        <v>6.879412161042652</v>
       </c>
       <c r="G106" t="n">
         <v>0.4026174994879254</v>
       </c>
       <c r="H106" t="n">
-        <v>4.696410910174022</v>
+        <v>4.696410910174029</v>
       </c>
       <c r="I106" t="n">
-        <v>26.14373195327791</v>
+        <v>26.14373195327786</v>
       </c>
       <c r="J106" t="n">
         <v>0.4</v>
       </c>
       <c r="K106" t="n">
-        <v>5.210672537910132</v>
+        <v>5.210672537910126</v>
       </c>
       <c r="L106" t="n">
-        <v>14.66638237813964</v>
+        <v>14.66638237813966</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>197.5197333722285</v>
+        <v>197.5197333722272</v>
       </c>
       <c r="B107" t="n">
         <v>0</v>
@@ -4494,16 +4494,16 @@
         <v>0</v>
       </c>
       <c r="E107" t="n">
-        <v>7.036525823518709</v>
+        <v>7.036525823518712</v>
       </c>
       <c r="F107" t="n">
-        <v>6.87941216104239</v>
+        <v>6.879412161042471</v>
       </c>
       <c r="G107" t="n">
         <v>0.9261043454272662</v>
       </c>
       <c r="H107" t="n">
-        <v>4.378071981065519</v>
+        <v>4.378071981065517</v>
       </c>
       <c r="I107" t="n">
         <v>28.20731119596918</v>
@@ -4512,15 +4512,15 @@
         <v>0.9</v>
       </c>
       <c r="K107" t="n">
-        <v>4.726652454008943</v>
+        <v>4.726652454008947</v>
       </c>
       <c r="L107" t="n">
-        <v>16.20755001913633</v>
+        <v>16.20755001913632</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>6.834780035277051</v>
+        <v>6.83478003555356</v>
       </c>
       <c r="B108" t="n">
         <v>0</v>
@@ -4532,33 +4532,33 @@
         <v>0.1</v>
       </c>
       <c r="E108" t="n">
-        <v>6.128497937407318</v>
+        <v>6.12849793740546</v>
       </c>
       <c r="F108" t="n">
-        <v>7.904787369190159</v>
+        <v>7.904787369195323</v>
       </c>
       <c r="G108" t="n">
         <v>0</v>
       </c>
       <c r="H108" t="n">
-        <v>5.846909926368788</v>
+        <v>5.846909926368639</v>
       </c>
       <c r="I108" t="n">
-        <v>20.72742782212903</v>
+        <v>20.72742782212946</v>
       </c>
       <c r="J108" t="n">
         <v>0</v>
       </c>
       <c r="K108" t="n">
-        <v>6.810947385913783</v>
+        <v>6.810947385901413</v>
       </c>
       <c r="L108" t="n">
-        <v>11.16889058376146</v>
+        <v>11.16889058380164</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>5.274583490016099</v>
+        <v>5.27458349120156</v>
       </c>
       <c r="B109" t="n">
         <v>0</v>
@@ -4570,33 +4570,33 @@
         <v>0.2</v>
       </c>
       <c r="E109" t="n">
-        <v>6.054000358592873</v>
+        <v>6.054000358603711</v>
       </c>
       <c r="F109" t="n">
-        <v>8.002693397380355</v>
+        <v>8.002693397328384</v>
       </c>
       <c r="G109" t="n">
         <v>0</v>
       </c>
       <c r="H109" t="n">
-        <v>5.846909926368786</v>
+        <v>5.846909926368784</v>
       </c>
       <c r="I109" t="n">
-        <v>20.72742782212903</v>
+        <v>20.72742782212904</v>
       </c>
       <c r="J109" t="n">
         <v>0</v>
       </c>
       <c r="K109" t="n">
-        <v>6.810947385909925</v>
+        <v>6.810947385874167</v>
       </c>
       <c r="L109" t="n">
-        <v>11.16889058379427</v>
+        <v>11.16889058380461</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>3.910921536253885</v>
+        <v>3.910921536759576</v>
       </c>
       <c r="B110" t="n">
         <v>0</v>
@@ -4608,33 +4608,33 @@
         <v>0.3</v>
       </c>
       <c r="E110" t="n">
-        <v>5.995457690847346</v>
+        <v>5.995457690830439</v>
       </c>
       <c r="F110" t="n">
-        <v>8.081355488661039</v>
+        <v>8.081355488716024</v>
       </c>
       <c r="G110" t="n">
         <v>0</v>
       </c>
       <c r="H110" t="n">
-        <v>5.84690992636879</v>
+        <v>5.846909926366481</v>
       </c>
       <c r="I110" t="n">
-        <v>20.72742782212902</v>
+        <v>20.72742782213567</v>
       </c>
       <c r="J110" t="n">
         <v>0</v>
       </c>
       <c r="K110" t="n">
-        <v>6.810947385881176</v>
+        <v>6.81094738586947</v>
       </c>
       <c r="L110" t="n">
-        <v>11.16889058380283</v>
+        <v>11.1688905838009</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>2.692555536845356</v>
+        <v>2.692555536037152</v>
       </c>
       <c r="B111" t="n">
         <v>0</v>
@@ -4646,33 +4646,33 @@
         <v>0.4</v>
       </c>
       <c r="E111" t="n">
-        <v>5.947428973040711</v>
+        <v>5.947428973040716</v>
       </c>
       <c r="F111" t="n">
-        <v>8.147058427425245</v>
+        <v>8.147058427425241</v>
       </c>
       <c r="G111" t="n">
         <v>0</v>
       </c>
       <c r="H111" t="n">
-        <v>5.846909926359623</v>
+        <v>5.846909926368788</v>
       </c>
       <c r="I111" t="n">
-        <v>20.72742782229992</v>
+        <v>20.72742782212903</v>
       </c>
       <c r="J111" t="n">
         <v>0</v>
       </c>
       <c r="K111" t="n">
-        <v>6.810947385890646</v>
+        <v>6.81094738590721</v>
       </c>
       <c r="L111" t="n">
-        <v>11.1688905838042</v>
+        <v>11.16889058379658</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>-2.079471920009799</v>
+        <v>-2.079471919994657</v>
       </c>
       <c r="B112" t="n">
         <v>0</v>
@@ -4684,33 +4684,33 @@
         <v>0.9</v>
       </c>
       <c r="E112" t="n">
-        <v>5.788470958957247</v>
+        <v>5.788470958957248</v>
       </c>
       <c r="F112" t="n">
-        <v>8.372370077823835</v>
+        <v>8.372370077823833</v>
       </c>
       <c r="G112" t="n">
         <v>0</v>
       </c>
       <c r="H112" t="n">
-        <v>5.846909926368789</v>
+        <v>5.846909926359956</v>
       </c>
       <c r="I112" t="n">
-        <v>20.72742782212902</v>
+        <v>20.72742782230031</v>
       </c>
       <c r="J112" t="n">
         <v>0</v>
       </c>
       <c r="K112" t="n">
-        <v>6.810947385874627</v>
+        <v>6.81094738588172</v>
       </c>
       <c r="L112" t="n">
-        <v>11.16889058380216</v>
+        <v>11.16889058380803</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>27.62637003434606</v>
+        <v>27.62637003434565</v>
       </c>
       <c r="B113" t="n">
         <v>0</v>
@@ -4722,10 +4722,10 @@
         <v>0</v>
       </c>
       <c r="E113" t="n">
-        <v>6.229814680542392</v>
+        <v>6.229814680542388</v>
       </c>
       <c r="F113" t="n">
-        <v>7.775428450084743</v>
+        <v>7.775428450084746</v>
       </c>
       <c r="G113" t="n">
         <v>0.1</v>
@@ -4748,7 +4748,7 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>45.98878045746835</v>
+        <v>45.98878045746655</v>
       </c>
       <c r="B114" t="n">
         <v>0</v>
@@ -4760,33 +4760,33 @@
         <v>0</v>
       </c>
       <c r="E114" t="n">
-        <v>6.229814680542415</v>
+        <v>6.229814680542374</v>
       </c>
       <c r="F114" t="n">
-        <v>7.775428450084248</v>
+        <v>7.775428450084835</v>
       </c>
       <c r="G114" t="n">
         <v>0.2</v>
       </c>
       <c r="H114" t="n">
-        <v>5.582196107608238</v>
+        <v>5.582196107608262</v>
       </c>
       <c r="I114" t="n">
-        <v>21.75916478669942</v>
+        <v>21.75916478669934</v>
       </c>
       <c r="J114" t="n">
         <v>0.1861872028258322</v>
       </c>
       <c r="K114" t="n">
-        <v>6.311575079575896</v>
+        <v>6.311575079575875</v>
       </c>
       <c r="L114" t="n">
-        <v>12.06536120701531</v>
+        <v>12.06536120701534</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>66.10333155687294</v>
+        <v>66.10333155687472</v>
       </c>
       <c r="B115" t="n">
         <v>0</v>
@@ -4798,33 +4798,33 @@
         <v>0</v>
       </c>
       <c r="E115" t="n">
-        <v>6.229814680542388</v>
+        <v>6.229814680542418</v>
       </c>
       <c r="F115" t="n">
-        <v>7.775428450084738</v>
+        <v>7.775428450084294</v>
       </c>
       <c r="G115" t="n">
         <v>0.3</v>
       </c>
       <c r="H115" t="n">
-        <v>5.467817013843073</v>
+        <v>5.467817013843058</v>
       </c>
       <c r="I115" t="n">
-        <v>22.23836450104402</v>
+        <v>22.23836450104408</v>
       </c>
       <c r="J115" t="n">
         <v>0.2724584114361717</v>
       </c>
       <c r="K115" t="n">
-        <v>6.134000054261062</v>
+        <v>6.134000054261064</v>
       </c>
       <c r="L115" t="n">
-        <v>12.42013818746446</v>
+        <v>12.42013818746445</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>87.92605840786248</v>
+        <v>87.92605840786152</v>
       </c>
       <c r="B116" t="n">
         <v>0</v>
@@ -4836,33 +4836,33 @@
         <v>0</v>
       </c>
       <c r="E116" t="n">
-        <v>6.229814680542417</v>
+        <v>6.229814680542386</v>
       </c>
       <c r="F116" t="n">
-        <v>7.775428450084322</v>
+        <v>7.775428450084768</v>
       </c>
       <c r="G116" t="n">
         <v>0.4</v>
       </c>
       <c r="H116" t="n">
-        <v>5.366971155165505</v>
+        <v>5.366971155165527</v>
       </c>
       <c r="I116" t="n">
-        <v>22.67925293210372</v>
+        <v>22.67925293210364</v>
       </c>
       <c r="J116" t="n">
         <v>0.3709916581317118</v>
       </c>
       <c r="K116" t="n">
-        <v>5.961526264742207</v>
+        <v>5.961526264742172</v>
       </c>
       <c r="L116" t="n">
-        <v>12.78546215459656</v>
+        <v>12.7854621545966</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>197.758045242448</v>
+        <v>197.7580452424492</v>
       </c>
       <c r="B117" t="n">
         <v>0</v>
@@ -4874,10 +4874,10 @@
         <v>0</v>
       </c>
       <c r="E117" t="n">
-        <v>6.229814680542415</v>
+        <v>6.229814680542383</v>
       </c>
       <c r="F117" t="n">
-        <v>7.775428450084292</v>
+        <v>7.775428450084793</v>
       </c>
       <c r="G117" t="n">
         <v>0.9</v>
@@ -4886,16 +4886,16 @@
         <v>5.013853272390429</v>
       </c>
       <c r="I117" t="n">
-        <v>24.37626844442449</v>
+        <v>24.3762684444245</v>
       </c>
       <c r="J117" t="n">
         <v>0.9187962143520164</v>
       </c>
       <c r="K117" t="n">
-        <v>5.375148878582299</v>
+        <v>5.375148878582295</v>
       </c>
       <c r="L117" t="n">
-        <v>14.20800890067435</v>
+        <v>14.20800890067436</v>
       </c>
     </row>
     <row r="118">
@@ -4912,33 +4912,33 @@
         <v>0</v>
       </c>
       <c r="E118" t="n">
-        <v>6.229814680542383</v>
+        <v>6.229814680542413</v>
       </c>
       <c r="F118" t="n">
-        <v>7.775428450084793</v>
+        <v>7.775428450084306</v>
       </c>
       <c r="G118" t="n">
         <v>0.1247653346366633</v>
       </c>
       <c r="H118" t="n">
-        <v>5.677040887610818</v>
+        <v>5.677040887610817</v>
       </c>
       <c r="I118" t="n">
-        <v>21.37759753844515</v>
+        <v>21.37759753844516</v>
       </c>
       <c r="J118" t="n">
         <v>0.1</v>
       </c>
       <c r="K118" t="n">
-        <v>6.523361592502432</v>
+        <v>6.523361592502427</v>
       </c>
       <c r="L118" t="n">
-        <v>11.66804559417191</v>
+        <v>11.66804559417192</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>48.00714090231821</v>
+        <v>48.00714090231396</v>
       </c>
       <c r="B119" t="n">
         <v>0</v>
@@ -4950,33 +4950,33 @@
         <v>0</v>
       </c>
       <c r="E119" t="n">
-        <v>6.229814680542414</v>
+        <v>6.229814680542411</v>
       </c>
       <c r="F119" t="n">
-        <v>7.775428450084282</v>
+        <v>7.775428450084238</v>
       </c>
       <c r="G119" t="n">
         <v>0.2063981465460308</v>
       </c>
       <c r="H119" t="n">
-        <v>5.574467231081983</v>
+        <v>5.574467231081984</v>
       </c>
       <c r="I119" t="n">
-        <v>21.79087610485098</v>
+        <v>21.79087610485097</v>
       </c>
       <c r="J119" t="n">
         <v>0.2</v>
       </c>
       <c r="K119" t="n">
-        <v>6.280953943054494</v>
+        <v>6.28095394305458</v>
       </c>
       <c r="L119" t="n">
-        <v>12.12507452459406</v>
+        <v>12.12507452459397</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>70.34975053173936</v>
+        <v>70.34975053170132</v>
       </c>
       <c r="B120" t="n">
         <v>0</v>
@@ -4988,33 +4988,33 @@
         <v>0</v>
       </c>
       <c r="E120" t="n">
-        <v>6.229814680542414</v>
+        <v>6.229814680542418</v>
       </c>
       <c r="F120" t="n">
-        <v>7.775428450084324</v>
+        <v>7.775428450084251</v>
       </c>
       <c r="G120" t="n">
         <v>0.3137697936590399</v>
       </c>
       <c r="H120" t="n">
-        <v>5.453144591001693</v>
+        <v>5.453144591001646</v>
       </c>
       <c r="I120" t="n">
-        <v>22.30141150939614</v>
+        <v>22.30141150939633</v>
       </c>
       <c r="J120" t="n">
         <v>0.3</v>
       </c>
       <c r="K120" t="n">
-        <v>6.083014358416881</v>
+        <v>6.083014358417758</v>
       </c>
       <c r="L120" t="n">
-        <v>12.52592282596386</v>
+        <v>12.52592282596257</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>90.85820507627585</v>
+        <v>90.85820507636862</v>
       </c>
       <c r="B121" t="n">
         <v>0</v>
@@ -5026,33 +5026,33 @@
         <v>0</v>
       </c>
       <c r="E121" t="n">
-        <v>6.229814680542382</v>
+        <v>6.229814680542388</v>
       </c>
       <c r="F121" t="n">
-        <v>7.775428450084776</v>
+        <v>7.775428450084751</v>
       </c>
       <c r="G121" t="n">
         <v>0.4026174994879254</v>
       </c>
       <c r="H121" t="n">
-        <v>5.364503824149426</v>
+        <v>5.364503824148882</v>
       </c>
       <c r="I121" t="n">
-        <v>22.69026561983227</v>
+        <v>22.69026561983405</v>
       </c>
       <c r="J121" t="n">
         <v>0.4</v>
       </c>
       <c r="K121" t="n">
-        <v>5.916680425885447</v>
+        <v>5.916680425885118</v>
       </c>
       <c r="L121" t="n">
-        <v>12.8840308499482</v>
+        <v>12.8840308499487</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>199.6739991890043</v>
+        <v>199.6739991890056</v>
       </c>
       <c r="B122" t="n">
         <v>0</v>
@@ -5064,10 +5064,10 @@
         <v>0</v>
       </c>
       <c r="E122" t="n">
-        <v>6.22981468054238</v>
+        <v>6.229814680542413</v>
       </c>
       <c r="F122" t="n">
-        <v>7.7754284500848</v>
+        <v>7.77542845008428</v>
       </c>
       <c r="G122" t="n">
         <v>0.9261043454272662</v>
@@ -5076,16 +5076,16 @@
         <v>5.000219964684943</v>
       </c>
       <c r="I122" t="n">
-        <v>24.44707451116663</v>
+        <v>24.44707451116664</v>
       </c>
       <c r="J122" t="n">
         <v>0.9</v>
       </c>
       <c r="K122" t="n">
-        <v>5.389450425310828</v>
+        <v>5.389450425310831</v>
       </c>
       <c r="L122" t="n">
-        <v>14.16951723043</v>
+        <v>14.16951723042999</v>
       </c>
     </row>
     <row r="123">
@@ -5102,7 +5102,7 @@
         <v>0</v>
       </c>
       <c r="E123" t="n">
-        <v>7.837064168615003</v>
+        <v>7.837064168615002</v>
       </c>
       <c r="F123" t="n">
         <v>6.173805682149559</v>
@@ -5120,7 +5120,7 @@
         <v>0.1</v>
       </c>
       <c r="K123" t="n">
-        <v>3.770437980766415</v>
+        <v>3.770437980766414</v>
       </c>
       <c r="L123" t="n">
         <v>20.4814558693205</v>
@@ -5140,19 +5140,19 @@
         <v>0</v>
       </c>
       <c r="E124" t="n">
-        <v>7.837064168615002</v>
+        <v>7.837064168614999</v>
       </c>
       <c r="F124" t="n">
-        <v>6.173805682149557</v>
+        <v>6.173805682149541</v>
       </c>
       <c r="G124" t="n">
         <v>0.1701643100102089</v>
       </c>
       <c r="H124" t="n">
-        <v>4.244175767458287</v>
+        <v>4.244175767458285</v>
       </c>
       <c r="I124" t="n">
-        <v>29.18131136449999</v>
+        <v>29.1813113645</v>
       </c>
       <c r="J124" t="n">
         <v>0.2</v>
@@ -5166,7 +5166,7 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>51.19915313046028</v>
+        <v>51.19915313046097</v>
       </c>
       <c r="B125" t="n">
         <v>90</v>
@@ -5178,10 +5178,10 @@
         <v>0</v>
       </c>
       <c r="E125" t="n">
-        <v>7.837064168614999</v>
+        <v>7.837064168615</v>
       </c>
       <c r="F125" t="n">
-        <v>6.173805682149546</v>
+        <v>6.173805682149554</v>
       </c>
       <c r="G125" t="n">
         <v>0.3214442565952542</v>
@@ -5190,21 +5190,21 @@
         <v>4.093997882615534</v>
       </c>
       <c r="I125" t="n">
-        <v>30.3619160937488</v>
+        <v>30.36191609374881</v>
       </c>
       <c r="J125" t="n">
         <v>0.3</v>
       </c>
       <c r="K125" t="n">
-        <v>3.630536246129327</v>
+        <v>3.630536246129323</v>
       </c>
       <c r="L125" t="n">
-        <v>21.30839062991481</v>
+        <v>21.30839062991482</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>58.88742559902328</v>
+        <v>58.88742559902227</v>
       </c>
       <c r="B126" t="n">
         <v>90</v>
@@ -5219,30 +5219,30 @@
         <v>7.837064168615</v>
       </c>
       <c r="F126" t="n">
-        <v>6.17380568214956</v>
+        <v>6.173805682149554</v>
       </c>
       <c r="G126" t="n">
         <v>0.3720151345183279</v>
       </c>
       <c r="H126" t="n">
-        <v>4.053242978902852</v>
+        <v>4.053242978902857</v>
       </c>
       <c r="I126" t="n">
-        <v>30.69998519193069</v>
+        <v>30.69998519193065</v>
       </c>
       <c r="J126" t="n">
         <v>0.4</v>
       </c>
       <c r="K126" t="n">
-        <v>3.586463213376641</v>
+        <v>3.586463213376665</v>
       </c>
       <c r="L126" t="n">
-        <v>21.58328154599323</v>
+        <v>21.58328154599474</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>122.9848839959848</v>
+        <v>122.9848839960663</v>
       </c>
       <c r="B127" t="n">
         <v>90</v>
@@ -5254,33 +5254,33 @@
         <v>0</v>
       </c>
       <c r="E127" t="n">
-        <v>7.837064168615003</v>
+        <v>7.837064168615002</v>
       </c>
       <c r="F127" t="n">
-        <v>6.173805682149572</v>
+        <v>6.173805682149539</v>
       </c>
       <c r="G127" t="n">
         <v>0.9137793267857967</v>
       </c>
       <c r="H127" t="n">
-        <v>3.761181232691156</v>
+        <v>3.761181232691152</v>
       </c>
       <c r="I127" t="n">
-        <v>33.37985343681321</v>
+        <v>33.37985343681326</v>
       </c>
       <c r="J127" t="n">
         <v>0.9</v>
       </c>
       <c r="K127" t="n">
-        <v>3.453741272603847</v>
+        <v>3.45374127260206</v>
       </c>
       <c r="L127" t="n">
-        <v>22.45695698888139</v>
+        <v>22.45695698889998</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>1.835788085431368</v>
+        <v>1.835788085108026</v>
       </c>
       <c r="B128" t="n">
         <v>90</v>
@@ -5292,33 +5292,33 @@
         <v>0</v>
       </c>
       <c r="E128" t="n">
-        <v>9.699347069291392</v>
+        <v>9.699347069291379</v>
       </c>
       <c r="F128" t="n">
-        <v>4.985069224042763</v>
+        <v>4.985069224042773</v>
       </c>
       <c r="G128" t="n">
         <v>0.1189512132472919</v>
       </c>
       <c r="H128" t="n">
-        <v>2.681662652113733</v>
+        <v>2.681662652128345</v>
       </c>
       <c r="I128" t="n">
-        <v>50.50392244803923</v>
+        <v>50.50392244784169</v>
       </c>
       <c r="J128" t="n">
         <v>0.1</v>
       </c>
       <c r="K128" t="n">
-        <v>1.908379287040441</v>
+        <v>1.90837928704069</v>
       </c>
       <c r="L128" t="n">
-        <v>43.73432903618903</v>
+        <v>43.73432903617852</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>2.634739230819063</v>
+        <v>2.634739230834278</v>
       </c>
       <c r="B129" t="n">
         <v>90</v>
@@ -5330,33 +5330,33 @@
         <v>0</v>
       </c>
       <c r="E129" t="n">
-        <v>9.699347069291383</v>
+        <v>9.699347069291399</v>
       </c>
       <c r="F129" t="n">
-        <v>4.985069224042769</v>
+        <v>4.985069224042785</v>
       </c>
       <c r="G129" t="n">
         <v>0.1701643100102089</v>
       </c>
       <c r="H129" t="n">
-        <v>2.675665367384411</v>
+        <v>2.675665367384082</v>
       </c>
       <c r="I129" t="n">
-        <v>50.65999279092324</v>
+        <v>50.65999279091609</v>
       </c>
       <c r="J129" t="n">
         <v>0.2</v>
       </c>
       <c r="K129" t="n">
-        <v>1.904998512896706</v>
+        <v>1.904998512780959</v>
       </c>
       <c r="L129" t="n">
-        <v>43.83169431140891</v>
+        <v>43.83169431849718</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>4.564451747701021</v>
+        <v>4.564451747724794</v>
       </c>
       <c r="B130" t="n">
         <v>90</v>
@@ -5368,33 +5368,33 @@
         <v>0</v>
       </c>
       <c r="E130" t="n">
-        <v>9.699347069291406</v>
+        <v>9.699347069291395</v>
       </c>
       <c r="F130" t="n">
-        <v>4.98506922404275</v>
+        <v>4.985069224042761</v>
       </c>
       <c r="G130" t="n">
         <v>0.3214442565952542</v>
       </c>
       <c r="H130" t="n">
-        <v>2.65998867903058</v>
+        <v>2.659988679030274</v>
       </c>
       <c r="I130" t="n">
-        <v>51.07378872710613</v>
+        <v>51.07378872710795</v>
       </c>
       <c r="J130" t="n">
         <v>0.3</v>
       </c>
       <c r="K130" t="n">
-        <v>1.901669738753149</v>
+        <v>1.90166973875314</v>
       </c>
       <c r="L130" t="n">
-        <v>43.92805650531952</v>
+        <v>43.92805650531964</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>5.247608665199103</v>
+        <v>5.247608665200418</v>
       </c>
       <c r="B131" t="n">
         <v>90</v>
@@ -5406,33 +5406,33 @@
         <v>0</v>
       </c>
       <c r="E131" t="n">
-        <v>9.699347069291386</v>
+        <v>9.69934706929139</v>
       </c>
       <c r="F131" t="n">
-        <v>4.98506922404277</v>
+        <v>4.985069224042777</v>
       </c>
       <c r="G131" t="n">
         <v>0.3720151345183279</v>
       </c>
       <c r="H131" t="n">
-        <v>2.6552967046603</v>
+        <v>2.655296704660302</v>
       </c>
       <c r="I131" t="n">
-        <v>51.19931357277213</v>
+        <v>51.19931357277207</v>
       </c>
       <c r="J131" t="n">
         <v>0.4</v>
       </c>
       <c r="K131" t="n">
-        <v>1.898391433030046</v>
+        <v>1.898391433026318</v>
       </c>
       <c r="L131" t="n">
-        <v>44.02344164232167</v>
+        <v>44.02344164232335</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>10.86255706230083</v>
+        <v>10.86255706230495</v>
       </c>
       <c r="B132" t="n">
         <v>90</v>
@@ -5444,28 +5444,28 @@
         <v>0</v>
       </c>
       <c r="E132" t="n">
-        <v>9.699347069291388</v>
+        <v>9.699347069291385</v>
       </c>
       <c r="F132" t="n">
-        <v>4.985069224042767</v>
+        <v>4.985069224042773</v>
       </c>
       <c r="G132" t="n">
         <v>0.9137793267857967</v>
       </c>
       <c r="H132" t="n">
-        <v>2.615721871101734</v>
+        <v>2.615721871101633</v>
       </c>
       <c r="I132" t="n">
-        <v>52.29043361348931</v>
+        <v>52.29043361349095</v>
       </c>
       <c r="J132" t="n">
         <v>0.9</v>
       </c>
       <c r="K132" t="n">
-        <v>1.882707929980548</v>
+        <v>1.882707929980482</v>
       </c>
       <c r="L132" t="n">
-        <v>44.48654708292874</v>
+        <v>44.48654708293421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>